<commit_message>
Aplica nome público, prazos e vagas do Encontro nº 02 (AI-002)
DEC-013: TECHNE Talks · Encontro nº 02 nos textos; material de apoio até 21/09 e ensaio no começo de outubro; Arthur envia os links e acompanha as inscrições com Henrique; restrição alimentar e limite de 20 no formulário de inscrição. Checklist com 40 tarefas.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardápio" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$44</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,7 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Technetalks — checklist</t>
+          <t>TECHNE Talks · Encontro nº 02 — checklist</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
@@ -678,7 +678,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="75" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>35</v>
       </c>
@@ -707,7 +707,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Ajustes sugeridos em docs/evento/FORMULARIOS.md: perguntas de escolha ocultas?, telefone com país Brasil, obrigatórias, restrição alimentar, quem indicou, termo "Lorem ipsum" no Coatio.</t>
+          <t>Ajustes em docs/evento/FORMULARIOS.md: perguntas de escolha ocultas?, telefone com país Brasil, obrigatórias, restrição alimentar (lactose, doença celíaca/glúten), quem indicou, termo "Lorem ipsum" no Coatio.</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Até 16 inscritos: 20 no total menos 2 organizadores e 2 palestrantes; descontar quem vier como apoio.</t>
+          <t>Limite de 20 respostas: organizadores e palestrantes também se inscrevem (DEC-013). Apoio que almoçar sem se inscrever reduz o limite.</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
@@ -872,22 +872,22 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Pelos formulários. Base dos flyers 2 e 3.</t>
+          <t>As respostas chegam no forms.app de Arthur. Base dos flyers 2 e 3.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Adicionar as pessoas ao grupo do WhatsApp</t>
+          <t>Receber o material de apoio (slides) e uma pergunta para o quiz de cada palestrante</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -903,11 +903,15 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Material de apoio até 21/09, junto com título e sinopse (DEC-013).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -916,7 +920,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Primeiro disparo: nome, foto e descrição do grupo + flyer 1</t>
+          <t>Adicionar as pessoas ao grupo do WhatsApp</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -932,29 +936,25 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Abre as inscrições com o link do formulário, depois de aprovado.</t>
-        </is>
-      </c>
+      <c r="G15" s="4" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Registro</t>
+          <t>Divulgação</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Convidar Guilherme Reis para fotos e vídeos, com o flyer</t>
+          <t>Primeiro disparo: nome, foto e descrição do grupo + flyer 1</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
@@ -967,60 +967,64 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>A confirmar até ele aceitar.</t>
+          <t>Abre as inscrições com o link do formulário, depois de aprovado.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Registro</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Flyer 2 — palestra do VIRUS</t>
+          <t>Convidar Guilherme Reis para fotos e vídeos, com o flyer</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>A confirmar até ele aceitar.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Definir a tela principal: projetor e telão, ou TV</t>
+          <t>Arthur, Henrique, VIRUS e Coatio se inscreverem no formulário</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur, Henrique, VIRUS e Coatio</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>46292</v>
+        <v>46286</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -1029,13 +1033,13 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal.</t>
+          <t>Todos contam nas 20 vagas (DEC-013). Depois da aprovação do formulário.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -1044,7 +1048,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Flyer 3 — palestra do Coatio</t>
+          <t>Flyer 2 — palestra do VIRUS</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1053,7 +1057,7 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>46296</v>
+        <v>46291</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -1064,25 +1068,25 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
+          <t>Definir a tela principal: projetor e telão, ou TV</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>46298</v>
+        <v>46292</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -1091,31 +1095,31 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Prazo proposto nos formulários; confirmar junto com o ensaio presencial de 16/10.</t>
+          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Divulgação</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Separar as mesas de plástico extras, se a planta precisar</t>
+          <t>Flyer 3 — palestra do Coatio</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -1126,50 +1130,54 @@
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Testar notebook → cabo/adaptador → tela com material real</t>
+          <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G22" s="4" t="n"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado: ensaio no começo de outubro, gravação com roteiro até 03/10 (DEC-013).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Banner: arte e encomenda</t>
+          <t>Separar as mesas de plástico extras, se a planta precisar</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
@@ -1180,29 +1188,25 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Previsão R$ 60.</t>
-        </is>
-      </c>
+      <c r="G23" s="4" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Brinde: comprar 2 canecas</t>
+          <t>Testar notebook → cabo/adaptador → tela com material real</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
@@ -1213,29 +1217,25 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Previsão R$ 70.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
+      <c r="G24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="4" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Confirmar quem prepara e serve o almoço no dia</t>
+          <t>Ensaio com a tela escolhida</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>Arthur + Henrique + palestrantes</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
@@ -1246,25 +1246,29 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G25" s="4" t="n"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Começo de outubro, data a combinar com os palestrantes, junto com o teste da tela (nº 4) (DEC-013).</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
+          <t>Banner: arte e encomenda</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
@@ -1277,27 +1281,27 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Aba Cardápio.</t>
+          <t>Previsão R$ 60.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
+          <t>Brinde: comprar 2 canecas</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
@@ -1310,31 +1314,31 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Pãezinhos, assados e café.</t>
+          <t>Previsão R$ 70.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Flyer 4 — vagas acabando</t>
+          <t>Confirmar quem prepara e serve o almoço no dia</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -1345,25 +1349,25 @@
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Avaliar pedidos de convidados de fora do grupo</t>
+          <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>46305</v>
+        <v>46299</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
@@ -1372,31 +1376,31 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>A pessoa vem com alguém do grupo e também se inscreve.</t>
+          <t>Aba Cardápio.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
+          <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>46305</v>
+        <v>46299</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -1405,22 +1409,22 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Anotar o número na aba Cardápio.</t>
+          <t>Pãezinhos, assados e café.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="n">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Divulgação</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
+          <t>Flyer 4 — vagas acabando</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -1429,40 +1433,36 @@
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Uma vez por semana a partir de 21/09. Base do flyer 4 (vagas acabando).</t>
-        </is>
-      </c>
+      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
+          <t>Avaliar pedidos de convidados de fora do grupo</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -1471,31 +1471,31 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Só depois de 10/10.</t>
+          <t>A pessoa vem com alguém do grupo e também se inscreve.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="4" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Receber slides e uma pergunta para o quiz de cada palestrante</t>
+          <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>46309</v>
+        <v>46305</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -1504,31 +1504,31 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Os formulários pedem "materiais finais" em 21/09: confirmar se os slides passam para 21/09.</t>
+          <t>Anotar o número na aba Cardápio.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="4" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Dinâmicas</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Montar o quiz do QR code e o formulário de feedback</t>
+          <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>46309</v>
+        <v>46305</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -1537,31 +1537,31 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
+          <t>Uma vez por semana a partir de 21/09. Base do flyer 4 (vagas acabando).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Dinâmicas</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Preparar a dinâmica de integração da recepção</t>
+          <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -1570,51 +1570,55 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Aproximar quem estiver isolado e formar grupos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
+          <t>Só depois de 10/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="45" customHeight="1">
       <c r="A36" s="4" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Dinâmicas</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Preparar a pergunta de abertura da Mesa 360</t>
+          <t>Planejar opção sem lactose e sem glúten para quem informar restrição</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G36" s="4" t="n"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Lasanha, estrogonofe e pães têm glúten ou lactose. Doença celíaca exige evitar contaminação cruzada (forma e utensílios separados).</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="4" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Enviar lembrete privado aos inscritos com o endereço</t>
+          <t>Montar o quiz do QR code e o formulário de feedback</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -1623,65 +1627,73 @@
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G37" s="4" t="n"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="4" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
+          <t>Preparar a dinâmica de integração da recepção</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G38" s="4" t="n"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Aproximar quem estiver isolado e formar grupos.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="4" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Ensaio com a tela escolhida</t>
+          <t>Preparar a pergunta de abertura da Mesa 360</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Arthur + Henrique + palestrantes</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
@@ -1692,58 +1704,54 @@
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="4" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Divulgação</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
+          <t>Enviar lembrete privado aos inscritos com o endereço</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>Só depois de 10/10.</t>
-        </is>
-      </c>
+      <c r="G40" s="4" t="n"/>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="4" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Pós-evento</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Agradecer no grupo e compartilhar fotos e materiais autorizados</t>
+          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
@@ -1754,44 +1762,106 @@
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Só depois de 10/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Pós-evento</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Agradecer no grupo e compartilhar fotos e materiais autorizados</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Pós-evento</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Fechar o balanço com comprovantes e acertar a divisão</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E42" s="6" t="n">
+      <c r="E44" s="6" t="n">
         <v>46319</v>
       </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>Aba Orçamento.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G42">
+  <autoFilter ref="A4:G44">
     <sortState ref="A5:G36">
       <sortCondition ref="E4:E36"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A5:G42">
+  <conditionalFormatting sqref="A5:G44">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$F5="Feito"</formula>
     </cfRule>
@@ -1806,7 +1876,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A fazer,Em andamento,Aguardando aprovação,Feito,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Registra a inscrição simplificada e o backlog de formulários (AI-002)
DEC-014: inscrição só com nome, WhatsApp e e-mail, conferida contra a versão publicada; perguntas de perfil e relacionamento no backlog do formulário de feedback; restrição alimentar para as próximas edições.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -612,7 +611,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>34</v>
       </c>
@@ -641,7 +640,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>forms.app. Link em docs/evento/FORMULARIOS.md</t>
+          <t>Refeito em 14/09 (versão 2): só nome, WhatsApp e e-mail, obrigatórios (DEC-014). Link em docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
@@ -678,7 +677,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="75" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>35</v>
       </c>
@@ -707,7 +706,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Ajustes em docs/evento/FORMULARIOS.md: perguntas de escolha ocultas?, telefone com país Brasil, obrigatórias, restrição alimentar (lactose, doença celíaca/glúten), quem indicou, termo "Lorem ipsum" no Coatio.</t>
+          <t>Inscrição v2: marcar os 3 campos como obrigatórios, Brasil como país padrão, DDD, descrição, mensagem final e cores. Palestrantes: termo "Lorem ipsum" no Coatio, perguntas de escolha ocultas?, obrigatórias. Detalhes em docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="45" customHeight="1">
+    <row r="36" ht="30" customHeight="1">
       <c r="A36" s="4" t="n">
         <v>39</v>
       </c>
@@ -1598,16 +1597,16 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Lasanha, estrogonofe e pães têm glúten ou lactose. Doença celíaca exige evitar contaminação cruzada (forma e utensílios separados).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
+          <t>Restrição alimentar fica para as próximas edições (DEC-014).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="60" customHeight="1">
       <c r="A37" s="4" t="n">
         <v>28</v>
       </c>
@@ -1618,7 +1617,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Montar o quiz do QR code e o formulário de feedback</t>
+          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -1636,7 +1635,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
+          <t>docs/evento/SORTEIO_E_FEEDBACK.md + itens de relacionamento do backlog em FORMULARIOS.md. Enviar no encerramento por QR code ou depois por e-mail/WhatsApp.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registra o lancamento de 14/09 e o passo a passo de comunicacao (AI-002)
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -3,16 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roteiro" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orçamento" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardápio" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comunicação" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roteiro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orçamento" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardápio" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$38</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,10 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +62,20 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +92,16 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -89,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,14 +138,35 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDDEBF7"/>
+          <bgColor rgb="FFDDEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="1"/>
@@ -141,8 +188,25 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFDDEBF7"/>
-          <bgColor rgb="FFDDEBF7"/>
+          <fgColor rgb="00D9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00999999"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00C00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -508,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" customWidth="1" min="1" max="1"/>
@@ -537,7 +601,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Amarelo: preencher. Azul: aguardando aprovação. Prazo vencido sem 'Feito' fica vermelho. Datas de divulgação são propostas até o aceite.</t>
+          <t>Amarelo: preencher. Azul: aguardando aprovação. Prazo vencido sem 'Feito' fica vermelho. As mensagens e as peças de divulgação ficam na aba Comunicação.</t>
         </is>
       </c>
     </row>
@@ -580,7 +644,7 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -589,91 +653,91 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Criar os formulários online dos palestrantes (VIRUS e Coatio)</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+          <t>Enviar o questionário aos dois palestrantes</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="20" t="n">
         <v>46279</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>forms.app. Links em docs/evento/FORMULARIOS.md</t>
+          <t>Links dos dois questionários enviados em 14/09 (DEC-015). docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Criar o formulário online de inscrição</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+          <t>Criar os formulários online dos palestrantes (VIRUS e Coatio)</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="20" t="n">
         <v>46279</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Refeito em 14/09 (versão 2): só nome, WhatsApp e e-mail, obrigatórios (DEC-014). Link em docs/evento/FORMULARIOS.md</t>
+          <t>forms.app. Links em docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="4" t="n">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Enviar o questionário aos dois palestrantes</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+          <t>Criar o formulário online de inscrição</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Aguardando aprovação</t>
+      <c r="E7" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Formulários online criados por Arthur em 14/09 (VIRUS e Coatio). Enviar os links só após a aprovação (nº 35). docs/evento/FORMULARIOS.md</t>
+          <t>Refeito em 14/09 (versão 2): só nome, WhatsApp e e-mail, obrigatórios (DEC-014). Link em docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
@@ -691,193 +755,193 @@
           <t>Revisar e aprovar os 3 formulários antes de enviar ou divulgar</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="20" t="n">
         <v>46281</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Aguardando aprovação</t>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Inscrição v2: marcar os 3 campos como obrigatórios, Brasil como país padrão, DDD, descrição, mensagem final e cores. Palestrantes: termo "Lorem ipsum" no Coatio, perguntas de escolha ocultas?, obrigatórias. Detalhes em docs/evento/FORMULARIOS.md</t>
+          <t>Aprovados na prática em 14/09: questionários enviados e inscrição divulgada no lançamento (DEC-015). Os ajustes que faltam estão na tarefa 41.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="4" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Desenhar a planta em 3 versões (seca, com móveis, com móveis e pessoas) com os 20 lugares e disponibilizar</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+          <t>Configurar no formulário o encerramento em 10/10 e o limite de vagas</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>46284</v>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Telas → sofá → 2 mesas com cadeiras → 2 mesas de plástico extras; quadro de vidro móvel; lanche e café embaixo da escada.</t>
+          <t>Limite de 20 respostas: organizadores e palestrantes também se inscrevem (DEC-013). O formulário já está divulgado, então o encerramento e o limite precisam entrar agora.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="4" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Definir como será a inscrição (link ou lista)</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Feito</t>
+          <t>Arthur, Henrique, VIRUS e Coatio se inscreverem no formulário</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Arthur, Henrique, VIRUS e Coatio</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>46284</v>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Formulário de inscrição no forms.app, criado em 14/09. Divulgar só após a aprovação (nº 35). docs/evento/FORMULARIOS.md</t>
+          <t>Todos contam nas 20 vagas (DEC-013). Palestrantes até 19/09 (DEC-015).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="n">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Formulários</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fazer a arte dos flyers a partir dos textos</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+          <t>Aplicar os ajustes pendentes do formulário de inscrição, já em uso</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>46284</v>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>docs/evento/DIVULGACAO.md. Flyer 1 primeiro.</t>
+          <t>Campos obrigatórios, Brasil (+55), DDD, descrição, mensagem final e cores. Os três campos sem obrigatoriedade são o risco maior: dá para receber inscrição sem telefone. docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Configurar no formulário o encerramento em 10/10 e o limite de vagas</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
+          <t>Desenhar a planta em 3 versões (seca, com móveis, com móveis e pessoas) com os 20 lugares e disponibilizar</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="n">
         <v>46285</v>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Limite de 20 respostas: organizadores e palestrantes também se inscrevem (DEC-013). Apoio que almoçar sem se inscrever reduz o limite.</t>
+          <t>Telas → sofá → 2 mesas com cadeiras → 2 mesas de plástico extras; quadro de vidro móvel; lanche e café embaixo da escada.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Divulgação</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Receber títulos e resumos das duas palestras</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
+          <t>Definir como será a inscrição (link ou lista)</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="E13" s="20" t="n">
+        <v>46285</v>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>As respostas chegam no forms.app de Arthur. Base dos flyers 2 e 3.</t>
+          <t>Formulário de inscrição no forms.app, criado em 14/09 e divulgado no lançamento do mesmo dia (DEC-015). docs/evento/FORMULARIOS.md</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -886,469 +950,481 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Receber o material de apoio (slides) e uma pergunta para o quiz de cada palestrante</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
+          <t>Receber títulos e resumos das duas palestras</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="n">
         <v>46286</v>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Material de apoio até 21/09, junto com título e sinopse (DEC-013).</t>
+          <t>Título, sinopse e minibio pelo formulário de cada palestrante. Base das peças 3 e 4. A cobrança está na aba Comunicação.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Adicionar as pessoas ao grupo do WhatsApp</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="n"/>
+          <t>Definir a tela principal: projetor e telão, ou TV</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>46292</v>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Primeiro disparo: nome, foto e descrição do grupo + flyer 1</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
+          <t>Receber o rascunho inicial do material de apoio e uma pergunta para o quiz de cada palestrante</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Abre as inscrições com o link do formulário, depois de aprovado.</t>
+          <t>Rascunho até 28/09; versão final e gravação do ensaio até 03/10 (DEC-015).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Registro</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Convidar Guilherme Reis para fotos e vídeos, com o flyer</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
+          <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>A confirmar até ele aceitar.</t>
+          <t>Ensaio no começo de outubro, gravação com roteiro até 03/10 (DEC-013 e DEC-015).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Arthur, Henrique, VIRUS e Coatio se inscreverem no formulário</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Arthur, Henrique, VIRUS e Coatio</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Todos contam nas 20 vagas (DEC-013). Depois da aprovação do formulário.</t>
-        </is>
-      </c>
+          <t>Separar as mesas de plástico extras, se a planta precisar</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Flyer 2 — palestra do VIRUS</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>46291</v>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="n"/>
+          <t>Testar notebook → cabo/adaptador → tela com material real</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Definir a tela principal: projetor e telão, ou TV</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>46292</v>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
+          <t>Ensaio com a tela escolhida</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique + palestrantes</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal.</t>
+          <t>Começo de outubro, data a combinar com os palestrantes, junto com o teste da tela (nº 4) (DEC-013).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Flyer 3 — palestra do Coatio</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
+          <t>Banner: arte e encomenda</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="n"/>
+      <c r="E21" s="20" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Previsão R$ 60.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
+          <t>Brinde: comprar 2 canecas</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="E22" s="20" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Confirmado: ensaio no começo de outubro, gravação com roteiro até 03/10 (DEC-013).</t>
+          <t>Previsão R$ 70.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Separar as mesas de plástico extras, se a planta precisar</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
+          <t>Confirmar quem prepara e serve o almoço no dia</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="20" t="n">
         <v>46299</v>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="n"/>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Testar notebook → cabo/adaptador → tela com material real</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
+          <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="n">
         <v>46299</v>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n"/>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Aba Cardápio.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="4" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Ensaio com a tela escolhida</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique + palestrantes</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n">
+          <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="n">
         <v>46299</v>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Começo de outubro, data a combinar com os palestrantes, junto com o teste da tela (nº 4) (DEC-013).</t>
+          <t>Pãezinhos, assados e café.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Banner: arte e encomenda</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
+          <t>Avaliar pedidos de convidados de fora do grupo</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Previsão R$ 60.</t>
+          <t>A pessoa vem com alguém do grupo e também se inscreve.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Brinde: comprar 2 canecas</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
+          <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Previsão R$ 70.</t>
+          <t>Anotar o número na aba Cardápio.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Inscrições</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Confirmar quem prepara e serve o almoço no dia</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n"/>
+          <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Uma vez por semana a partir do lançamento de 14/09. Base da peça 5 (últimas vagas).</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -1357,31 +1433,31 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
+          <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="E29" s="20" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Aba Cardápio.</t>
+          <t>Só depois de 10/10.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
@@ -1390,159 +1466,155 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
+          <t>Planejar opção sem lactose e sem glúten para quem informar restrição</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="E30" s="20" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Pãezinhos, assados e café.</t>
+          <t>Restrição alimentar fica para as próximas edições (DEC-014 e DEC-015). Risco aceito: o cardápio tem glúten e lactose em quase tudo.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Divulgação</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Flyer 4 — vagas acabando</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
+          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n">
-        <v>46301</v>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="n"/>
+      <c r="E31" s="20" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>docs/evento/SORTEIO_E_FEEDBACK.md + itens de relacionamento do backlog em FORMULARIOS.md. Enviar no encerramento por QR code ou depois por e-mail/WhatsApp.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Avaliar pedidos de convidados de fora do grupo</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
+          <t>Preparar a dinâmica de integração da recepção</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="E32" s="20" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>A pessoa vem com alguém do grupo e também se inscreve.</t>
+          <t>Aproximar quem estiver isolado e formar grupos.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="4" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
+          <t>Preparar a pergunta de abertura da Mesa 360</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Anotar o número na aba Cardápio.</t>
-        </is>
-      </c>
+      <c r="E33" s="20" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="4" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Inscrições</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Uma vez por semana a partir de 21/09. Base do flyer 4 (vagas acabando).</t>
-        </is>
-      </c>
+          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
@@ -1551,18 +1623,18 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
+          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="E35" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
@@ -1575,308 +1647,68 @@
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="4" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Pós-evento</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Planejar opção sem lactose e sem glúten para quem informar restrição</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Não se aplica</t>
+          <t>Fechar o balanço com comprovantes e acertar a divisão</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E36" s="20" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Restrição alimentar fica para as próximas edições (DEC-014).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Dinâmicas</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md + itens de relacionamento do backlog em FORMULARIOS.md. Enviar no encerramento por QR code ou depois por e-mail/WhatsApp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Dinâmicas</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Preparar a dinâmica de integração da recepção</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>Aproximar quem estiver isolado e formar grupos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Dinâmicas</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Preparar a pergunta de abertura da Mesa 360</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Divulgação</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Enviar lembrete privado aos inscritos com o endereço</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>46310</v>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Espaço</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>Só depois de 10/10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Pós-evento</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Agradecer no grupo e compartilhar fotos e materiais autorizados</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>46315</v>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Pós-evento</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Fechar o balanço com comprovantes e acertar a divisão</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="n">
-        <v>46319</v>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
           <t>Aba Orçamento.</t>
         </is>
       </c>
     </row>
+    <row r="37" ht="60" customHeight="1"/>
+    <row r="38" ht="30" customHeight="1"/>
+    <row r="39" ht="30" customHeight="1"/>
+    <row r="40" ht="30" customHeight="1"/>
+    <row r="41" ht="30" customHeight="1"/>
+    <row r="42" ht="30" customHeight="1"/>
+    <row r="43" ht="30" customHeight="1"/>
+    <row r="44" ht="30" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A4:G44">
+  <autoFilter ref="A4:G36">
     <sortState ref="A5:G36">
       <sortCondition ref="E4:E36"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A5:G44">
-    <cfRule type="expression" priority="1" dxfId="2">
+  <conditionalFormatting sqref="A5:G36">
+    <cfRule type="expression" priority="5" dxfId="4">
       <formula>$F5="Feito"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="6" dxfId="5">
       <formula>$F5="Não se aplica"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="0">
+    <cfRule type="expression" priority="7" dxfId="6">
       <formula>AND($E5&lt;TODAY(),$F5&lt;&gt;"Feito",$F5&lt;&gt;"Não se aplica")</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="8" dxfId="7">
       <formula>$F5="Aguardando aprovação"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"A fazer,Em andamento,Aguardando aprovação,Feito,Não se aplica"</formula1>
+    <dataValidation sqref="F5:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1885,6 +1717,1525 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>TECHNE Talks · Encontro nº 02 — comunicação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Ordem padrão das mensagens, reutilizável nas próximas edições. Passo a passo e radar do que ainda falta comunicar: docs/evento/COMUNICACAO.md. Textos prontos: docs/evento/DIVULGACAO.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Amarelo: preencher. Prazo vencido sem 'Feito' fica vermelho. Quem envia é sempre um organizador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Fase</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Peça / mensagem</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Gatilho</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Canal</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Responsável</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Fechar a identidade: nome público, logo e paleta</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Data e local fechados</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>46277</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Escrever a descrição do grupo, a mensagem de lançamento e os textos das peças</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Identidade fechada</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Repositório</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>docs/evento/DIVULGACAO.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Criar e testar o formulário de inscrição</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Textos prontos</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>forms.app</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>docs/evento/FORMULARIOS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Produzir as artes das peças 1 (convite) e 2 (programação)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Textos aprovados</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Aprovar as artes e os textos finais</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Artes prontas</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Aprovação dos dois organizadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>1 · Lançamento</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Trocar nome, foto e descrição do grupo</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Nome: TΞKHNE Talks - 2ª Edição. Foto: logo do TECHNE Talks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>1 · Lançamento</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Restringir o grupo a mensagens de admins</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Antes do disparo</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Temporário e anunciado na mensagem de lançamento. Reabertura na peça nº 13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>1 · Lançamento</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Mensagem de lançamento + peças 1 e 2 + link de inscrição</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Grupo preparado</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Abre as inscrições. Os palestrantes não foram anunciados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>2 · Palestrantes</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Enviar o questionário a VIRUS e Coatio</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Formulário aprovado</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2 · Palestrantes</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Pedir aos palestrantes que se inscrevam no formulário</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Questionário enviado</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>46284</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Eles contam nas 20 vagas. Libera a cobrança do material.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>1 · Lançamento</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Convidar Guilherme Reis para registrar o dia, com a peça 1</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Peça 1 publicada</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Fica 'a confirmar' até ele aceitar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>1 · Lançamento</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Adicionar os convidados ao grupo</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Lançamento feito</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Pessoas próximas, de tecnologia ou de interesse genuíno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>3 · Sustentação</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Reabrir o grupo para todos</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Primeira rodada absorvida</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Encerra a fase só de admins. Texto pronto em DIVULGACAO.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>2 · Palestrantes</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Cobrar título, sinopse e minibio</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Inscrição confirmada</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Sem isso as peças 3 e 4 saem só com o tema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Produzir a arte da peça 3 (palestra 1)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Título recebido</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>3 · Sustentação</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Anúncio da palestra 1, com a peça 3</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Arte pronta</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>2 · Palestrantes</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Cobrar o rascunho inicial do material de apresentação</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Título recebido</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Rascunho, não versão final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Produzir a arte da peça 4 (palestra 2)</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Título recebido</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>3 · Sustentação</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Anúncio da palestra 2, com a peça 4</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Arte pronta</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>2 · Palestrantes</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Combinar o ensaio e cobrar a gravação com o roteiro</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Material em rascunho</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Junto com o teste da tela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>0 · Preparação</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Produzir a arte da peça 5 (últimas vagas)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Vagas em queda</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>3 · Sustentação</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Últimas vagas, com a peça 5</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Arte pronta</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>46301</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Precisa do número de vagas restantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>3 · Sustentação</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Aviso de encerramento das inscrições</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Data-limite</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Última chance de liberar vaga de quem desistir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>4 · Semana do evento</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Confirmar presença de cada inscrito</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Inscrições encerradas</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Base do quantitativo de comida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>4 · Semana do evento</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Lembrete final: endereço, horário, o que levar e registro de imagem</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Presença confirmada</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>O endereço já está na peça 1; o lembrete reforça e confirma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>4 · Semana do evento</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Confirmar roteiro e horários com os palestrantes</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Ensaio feito</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>5 · Dia</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Bom dia com endereço e horário de chegada</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Manhã do evento</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>5 · Dia</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Divulgar o QR code do quiz e conduzir o sorteio</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Mesa 360</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>No local</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>5 · Dia</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Divulgar o QR code do feedback no encerramento</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Encerramento</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>No local</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Agradecimento no grupo, no mesmo dia</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Fim do evento</t>
+        </is>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Publicar fotos e materiais autorizados</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Autorizações conferidas</t>
+        </is>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H35" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Só o que palestrantes e participantes autorizaram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Reenviar o feedback a quem não respondeu</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Respostas paradas</t>
+        </is>
+      </c>
+      <c r="E36" s="20" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H36" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Resultado do feedback e convite para a próxima edição</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Feedback consolidado</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H37" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Registrar os aprendizados de comunicação da edição</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Contas fechadas</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Repositório</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>O que mudar no passo a passo da próxima edição.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:I38"/>
+  <conditionalFormatting sqref="A5:I38">
+    <cfRule type="expression" priority="1" dxfId="4">
+      <formula>$H5="Feito"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="5">
+      <formula>$H5="Não se aplica"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="6">
+      <formula>AND($E5&lt;TODAY(),$H5&lt;&gt;"Feito",$H5&lt;&gt;"Não se aplica")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="7">
+      <formula>$H5="Aguardando aprovação"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2186,7 +3537,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2254,10 +3605,10 @@
           <t>Banner</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="C5" s="15" t="n"/>
+      <c r="C5" s="10" t="n"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Agora</t>
@@ -2272,10 +3623,10 @@
           <t>Brinde (2 canecas)</t>
         </is>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="C6" s="15" t="n"/>
+      <c r="C6" s="10" t="n"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Agora</t>
@@ -2290,10 +3641,10 @@
           <t>Almoço</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="9" t="n">
         <v>250</v>
       </c>
-      <c r="C7" s="15" t="n"/>
+      <c r="C7" s="10" t="n"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Depois de 10/10</t>
@@ -2308,10 +3659,10 @@
           <t>Lanche</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="C8" s="15" t="n"/>
+      <c r="C8" s="10" t="n"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Depois de 10/10</t>
@@ -2326,10 +3677,10 @@
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="C9" s="15" t="n"/>
+      <c r="C9" s="10" t="n"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Depois de 10/10</t>
@@ -2344,10 +3695,10 @@
           <t>Café</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="C10" s="15" t="n"/>
+      <c r="C10" s="10" t="n"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Depois de 10/10</t>
@@ -2362,18 +3713,18 @@
           <t>Soma</t>
         </is>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="12">
         <f>SUM(B5:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="12">
         <f>SUM(C5:C10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
     </row>
     <row r="13" ht="18.75" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
@@ -2381,8 +3732,8 @@
           <t>Balanço</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="14" t="n"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2390,10 +3741,10 @@
           <t>Previsão da edição</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="C14" s="14" t="n"/>
+      <c r="C14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2401,11 +3752,11 @@
           <t>Soma das categorias − previsão</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="9">
         <f>B11-B14</f>
         <v/>
       </c>
-      <c r="C15" s="14" t="n"/>
+      <c r="C15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2413,11 +3764,11 @@
           <t>Gasto real total</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="9">
         <f>C11</f>
         <v/>
       </c>
-      <c r="C16" s="14" t="n"/>
+      <c r="C16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2425,11 +3776,11 @@
           <t>Pago por Arthur</t>
         </is>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="9">
         <f>SUMIF(E5:E10,"Arthur",C5:C10)</f>
         <v/>
       </c>
-      <c r="C17" s="14" t="n"/>
+      <c r="C17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2437,11 +3788,11 @@
           <t>Pago por Henrique</t>
         </is>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="9">
         <f>SUMIF(E5:E10,"Henrique",C5:C10)</f>
         <v/>
       </c>
-      <c r="C18" s="14" t="n"/>
+      <c r="C18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2449,11 +3800,11 @@
           <t>Parte de cada um (metade)</t>
         </is>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="9">
         <f>C11/2</f>
         <v/>
       </c>
-      <c r="C19" s="14" t="n"/>
+      <c r="C19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2461,11 +3812,10 @@
           <t>Acerto: positivo = Henrique repassa a Arthur</t>
         </is>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="21">
         <f>B17-B19</f>
         <v/>
       </c>
-      <c r="C20" s="14" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2477,7 +3827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Aplica as confirmacoes de 15/09 do evento (AI-002)
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -798,12 +798,12 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Limite de 20 respostas: organizadores e palestrantes também se inscrevem (DEC-013). O formulário já está divulgado, então o encerramento e o limite precisam entrar agora.</t>
+          <t>Arthur mantém o formulário como está e faz o controle à mão: confere as inscrições, conta as 20 vagas e encerra a lista em 10/10 (DEC-016).</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Todos contam nas 20 vagas (DEC-013). Palestrantes até 19/09 (DEC-015).</t>
+          <t>Todos contam nas 20 vagas (DEC-013). Palestrantes até 19/09, confirmado em 15/09 (DEC-016).</t>
         </is>
       </c>
     </row>
@@ -864,12 +864,12 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Campos obrigatórios, Brasil (+55), DDD, descrição, mensagem final e cores. Os três campos sem obrigatoriedade são o risco maior: dá para receber inscrição sem telefone. docs/evento/FORMULARIOS.md</t>
+          <t>Ajustes do forms.app dispensados por Arthur em 15/09 (DEC-016). A tabela de conferência de FORMULARIOS.md fica como referência para a próxima edição.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Título, sinopse e minibio pelo formulário de cada palestrante. Base das peças 3 e 4. A cobrança está na aba Comunicação.</t>
+          <t>Título, sinopse e minibio até 21/09, confirmado em 15/09 (DEC-016). Base das peças 3 e 4; a cobrança está na aba Comunicação.</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Rascunho até 28/09; versão final e gravação do ensaio até 03/10 (DEC-015).</t>
+          <t>Rascunho até 28/09; versão final e gravação do ensaio até 03/10. Prazos confirmados em 15/09 (DEC-016).</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Ensaio no começo de outubro, gravação com roteiro até 03/10 (DEC-013 e DEC-015).</t>
+          <t>Ensaio no começo de outubro, gravação com roteiro até 03/10. Confirmado em 15/09 (DEC-016).</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E28" s="20" t="n">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Uma vez por semana a partir do lançamento de 14/09. Base da peça 5 (últimas vagas).</t>
+          <t>Contagem à mão, uma vez por semana a partir do lançamento de 14/09 (DEC-016). Base da peça 5 (últimas vagas).</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>docs/evento/FORMULARIOS.md</t>
+          <t>docs/evento/FORMULARIOS.md. Fica como está; vagas e encerramento controlados à mão (DEC-016).</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Nome: TΞKHNE Talks - 2ª Edição. Foto: logo do TECHNE Talks.</t>
+          <t>Nome padronizado com C em 15/09: TΞCHNE Talks - 2ª Edição. Foto: logo do TECHNE Talks.</t>
         </is>
       </c>
     </row>
@@ -2181,29 +2181,29 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>2 · Palestrantes</t>
+          <t>3 · Sustentação</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Pedir aos palestrantes que se inscrevam no formulário</t>
+          <t>Reabrir o grupo para todos</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Questionário enviado</t>
+          <t>Primeira rodada absorvida</t>
         </is>
       </c>
       <c r="E14" s="20" t="n">
-        <v>46284</v>
+        <v>46281</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
@@ -2218,31 +2218,31 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Eles contam nas 20 vagas. Libera a cobrança do material.</t>
+          <t>Encerra a fase só de admins, na noite de 16/09 (DEC-016). Texto pronto em DIVULGACAO.md.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>1 · Lançamento</t>
+          <t>2 · Palestrantes</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Convidar Guilherme Reis para registrar o dia, com a peça 1</t>
+          <t>Pedir aos palestrantes que se inscrevam no formulário</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Peça 1 publicada</t>
+          <t>Questionário enviado</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
@@ -2261,13 +2261,13 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Fica 'a confirmar' até ele aceitar.</t>
+          <t>Eles contam nas 20 vagas. Libera a cobrança do material.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
@@ -2276,12 +2276,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Adicionar os convidados ao grupo</t>
+          <t>Convidar Guilherme Reis para registrar o dia, com a peça 1</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Lançamento feito</t>
+          <t>Peça 1 publicada</t>
         </is>
       </c>
       <c r="E16" s="20" t="n">
@@ -2289,12 +2289,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="H16" s="14" t="inlineStr">
@@ -2304,27 +2304,27 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Pessoas próximas, de tecnologia ou de interesse genuíno.</t>
+          <t>Fica 'a confirmar' até ele aceitar.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>3 · Sustentação</t>
+          <t>1 · Lançamento</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Reabrir o grupo para todos</t>
+          <t>Adicionar os convidados ao grupo</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Primeira rodada absorvida</t>
+          <t>Lançamento feito</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Encerra a fase só de admins. Texto pronto em DIVULGACAO.md.</t>
+          <t>Pessoas próximas, de tecnologia ou de interesse genuíno.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registra as respostas do Coatio e prepara o anuncio (AI-002)
Coatio respondeu ao questionario em 23/09, fora do prazo e antes do
VIRUS. DEC-017 registra as respostas, o tema corrigido (bastidores da
construcao do Caranga, com demonstracao do piloto, no lugar de design
thinking e UI/UX) e as decisoes de Arthur: anunciar sem numerar a
palestra, encurtar o titulo para a arte e tratar a foto em p&b.

Novo docs/evento/RESPOSTAS_PALESTRANTES.md com as respostas na integra
e as pendencias. Peca 4 escrita para sair antes da peca 3, com mensagens
privadas de retorno ao Coatio e cobranca ao VIRUS. Planilha com 3 pecas
novas e 5 alteradas na aba Comunicacao.

As fotos tratadas ficaram fora do commit: o palestrante autorizou
divulgacao publica apenas mediante aprovacao, e o repositorio e publico.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$41</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="&quot;R$&quot; #,##0.00"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -939,7 +940,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>7</v>
       </c>
@@ -968,11 +969,11 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Título, sinopse e minibio até 21/09, confirmado em 15/09 (DEC-016). Base das peças 3 e 4; a cobrança está na aba Comunicação.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>Coatio entregou em 23/09, dois dias depois do prazo; VIRUS atrasado desde 21/09 (DEC-017). Respostas em docs/evento/RESPOSTAS_PALESTRANTES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>2</v>
       </c>
@@ -1001,7 +1002,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal.</t>
+          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal. O Coatio pediu projetor + HDMI e tem demonstração do piloto: avisar ele da decisão.</t>
         </is>
       </c>
     </row>
@@ -1722,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1841,7 +1842,7 @@
           <t>Feito</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -1966,7 +1967,7 @@
           <t>Feito</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -2177,7 +2178,7 @@
           <t>Feito</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -2390,13 +2391,13 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Sem isso as peças 3 e 4 saem só com o tema.</t>
+          <t>Coatio respondeu em 23/09, dois dias depois do prazo (DEC-017). VIRUS não respondeu; cobrança na peça 36.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -2405,7 +2406,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Produzir a arte da peça 3 (palestra 1)</t>
+          <t>Produzir a arte da peça 4 (palestra 2)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -2414,7 +2415,7 @@
         </is>
       </c>
       <c r="E19" s="20" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
@@ -2431,33 +2432,37 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Texto, foto tratada em p&amp;b e recorte 4:5 prontos em 23/09 (docs/evento/DIVULGACAO.md e outputs/AI-002/).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>3 · Sustentação</t>
+          <t>2 · Palestrantes</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Anúncio da palestra 1, com a peça 3</t>
+          <t>Confirmar com o Coatio o título curto, a foto tratada, os prazos e o plano B</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Arte pronta</t>
+          <t>Respostas recebidas</t>
         </is>
       </c>
       <c r="E20" s="20" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr">
@@ -2470,33 +2475,37 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Texto pronto em docs/evento/DIVULGACAO.md. A peça 4 não sai antes deste aval (DEC-017).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>2 · Palestrantes</t>
+          <t>3 · Sustentação</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Cobrar o rascunho inicial do material de apresentação</t>
+          <t>Anúncio do convidado confirmado (Coatio), com a peça 4</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Título recebido</t>
+          <t>Arte pronta</t>
         </is>
       </c>
       <c r="E21" s="20" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
@@ -2511,35 +2520,35 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Rascunho, não versão final.</t>
+          <t>Sai como convidado confirmado, sem numerar a palestra, porque o VIRUS ainda não respondeu (DEC-017).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>0 · Preparação</t>
+          <t>2 · Palestrantes</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Produzir a arte da peça 4 (palestra 2)</t>
+          <t>Cobrar o questionário do VIRUS e esclarecer "uso concorrente"</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Título recebido</t>
+          <t>Prazo vencido em 21/09</t>
         </is>
       </c>
       <c r="E22" s="20" t="n">
-        <v>46295</v>
+        <v>46291</v>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -2552,33 +2561,37 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Trava a peça 3 e o anúncio da palestra dele.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>3 · Sustentação</t>
+          <t>2 · Palestrantes</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Anúncio da palestra 2, com a peça 4</t>
+          <t>Avisar o Coatio da tela escolhida, projetor ou TV</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Arte pronta</t>
+          <t>Decisão de 27/09</t>
         </is>
       </c>
       <c r="E23" s="20" t="n">
-        <v>46296</v>
+        <v>46292</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
@@ -2591,11 +2604,15 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Ele pediu projetor + HDMI e tem demonstração do piloto (DEC-017).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -2604,16 +2621,16 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Combinar o ensaio e cobrar a gravação com o roteiro</t>
+          <t>Cobrar o rascunho inicial do material de apresentação</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Material em rascunho</t>
+          <t>Título recebido</t>
         </is>
       </c>
       <c r="E24" s="20" t="n">
-        <v>46298</v>
+        <v>46293</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
@@ -2632,13 +2649,13 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Junto com o teste da tela.</t>
+          <t>Rascunho, não versão final.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
@@ -2647,16 +2664,16 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Produzir a arte da peça 5 (últimas vagas)</t>
+          <t>Produzir a arte da peça 3 (palestra 1)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Vagas em queda</t>
+          <t>Título recebido</t>
         </is>
       </c>
       <c r="E25" s="20" t="n">
-        <v>46300</v>
+        <v>46295</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
@@ -2673,11 +2690,15 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Parada até o VIRUS responder. Trocou de data com a peça 4 (DEC-017).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
@@ -2686,7 +2707,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Últimas vagas, com a peça 5</t>
+          <t>Anúncio da palestra 1, com a peça 3</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -2695,7 +2716,7 @@
         </is>
       </c>
       <c r="E26" s="20" t="n">
-        <v>46301</v>
+        <v>46296</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
@@ -2714,40 +2735,40 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Precisa do número de vagas restantes.</t>
+          <t>Depende das respostas do VIRUS.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>3 · Sustentação</t>
+          <t>2 · Palestrantes</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Aviso de encerramento das inscrições</t>
+          <t>Combinar o ensaio e cobrar a gravação com o roteiro</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Data-limite</t>
+          <t>Material em rascunho</t>
         </is>
       </c>
       <c r="E27" s="20" t="n">
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
@@ -2757,40 +2778,40 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Última chance de liberar vaga de quem desistir.</t>
+          <t>Junto com o teste da tela.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>4 · Semana do evento</t>
+          <t>0 · Preparação</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Confirmar presença de cada inscrito</t>
+          <t>Produzir a arte da peça 5 (últimas vagas)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Inscrições encerradas</t>
+          <t>Vagas em queda</t>
         </is>
       </c>
       <c r="E28" s="20" t="n">
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H28" s="14" t="inlineStr">
@@ -2798,37 +2819,33 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Base do quantitativo de comida.</t>
-        </is>
-      </c>
+      <c r="I28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>4 · Semana do evento</t>
+          <t>3 · Sustentação</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Lembrete final: endereço, horário, o que levar e registro de imagem</t>
+          <t>Últimas vagas, com a peça 5</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Presença confirmada</t>
+          <t>Arte pronta</t>
         </is>
       </c>
       <c r="E29" s="20" t="n">
-        <v>46310</v>
+        <v>46301</v>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr">
@@ -2843,40 +2860,40 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>O endereço já está na peça 1; o lembrete reforça e confirma.</t>
+          <t>Precisa do número de vagas restantes.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>4 · Semana do evento</t>
+          <t>3 · Sustentação</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Confirmar roteiro e horários com os palestrantes</t>
+          <t>Aviso de encerramento das inscrições</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Ensaio feito</t>
+          <t>Data-limite</t>
         </is>
       </c>
       <c r="E30" s="20" t="n">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
@@ -2884,38 +2901,42 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>Última chance de liberar vaga de quem desistir.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>5 · Dia</t>
+          <t>4 · Semana do evento</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Bom dia com endereço e horário de chegada</t>
+          <t>Confirmar presença de cada inscrito</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Manhã do evento</t>
+          <t>Inscrições encerradas</t>
         </is>
       </c>
       <c r="E31" s="20" t="n">
-        <v>46312</v>
+        <v>46307</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
@@ -2923,38 +2944,42 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Base do quantitativo de comida.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>5 · Dia</t>
+          <t>4 · Semana do evento</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Divulgar o QR code do quiz e conduzir o sorteio</t>
+          <t>Lembrete final: endereço, horário, o que levar e registro de imagem</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Mesa 360</t>
+          <t>Presença confirmada</t>
         </is>
       </c>
       <c r="E32" s="20" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>No local</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
@@ -2964,40 +2989,40 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
+          <t>O endereço já está na peça 1; o lembrete reforça e confirma.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>5 · Dia</t>
+          <t>4 · Semana do evento</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Divulgar o QR code do feedback no encerramento</t>
+          <t>Confirmar roteiro e horários com os palestrantes</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Encerramento</t>
+          <t>Ensaio feito</t>
         </is>
       </c>
       <c r="E33" s="20" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>No local</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
@@ -3005,25 +3030,25 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>6 · Pós-evento</t>
+          <t>5 · Dia</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Agradecimento no grupo, no mesmo dia</t>
+          <t>Bom dia com endereço e horário de chegada</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Fim do evento</t>
+          <t>Manhã do evento</t>
         </is>
       </c>
       <c r="E34" s="20" t="n">
@@ -3044,33 +3069,33 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>6 · Pós-evento</t>
+          <t>5 · Dia</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Publicar fotos e materiais autorizados</t>
+          <t>Divulgar o QR code do quiz e conduzir o sorteio</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Autorizações conferidas</t>
+          <t>Mesa 360</t>
         </is>
       </c>
       <c r="E35" s="20" t="n">
-        <v>46315</v>
+        <v>46312</v>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>No local</t>
         </is>
       </c>
       <c r="G35" s="14" t="inlineStr">
@@ -3085,40 +3110,40 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Só o que palestrantes e participantes autorizaram.</t>
+          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>6 · Pós-evento</t>
+          <t>5 · Dia</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Reenviar o feedback a quem não respondeu</t>
+          <t>Divulgar o QR code do feedback no encerramento</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Respostas paradas</t>
+          <t>Encerramento</t>
         </is>
       </c>
       <c r="E36" s="20" t="n">
-        <v>46315</v>
+        <v>46312</v>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>No local</t>
         </is>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
@@ -3126,11 +3151,11 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
@@ -3139,16 +3164,16 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Resultado do feedback e convite para a próxima edição</t>
+          <t>Agradecimento no grupo, no mesmo dia</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Feedback consolidado</t>
+          <t>Fim do evento</t>
         </is>
       </c>
       <c r="E37" s="20" t="n">
-        <v>46319</v>
+        <v>46312</v>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
@@ -3157,7 +3182,7 @@
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
@@ -3165,54 +3190,175 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Publicar fotos e materiais autorizados</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Autorizações conferidas</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Só o que palestrantes e participantes autorizaram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Reenviar o feedback a quem não respondeu</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Respostas paradas</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Resultado do feedback e convite para a próxima edição</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Feedback consolidado</t>
+        </is>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H40" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>6 · Pós-evento</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Registrar os aprendizados de comunicação da edição</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>Contas fechadas</t>
         </is>
       </c>
-      <c r="E38" s="20" t="n">
+      <c r="E41" s="20" t="n">
         <v>46319</v>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>Repositório</t>
         </is>
       </c>
-      <c r="G38" s="14" t="inlineStr">
+      <c r="G41" s="14" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H38" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
         <is>
           <t>O que mudar no passo a passo da próxima edição.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I38"/>
-  <conditionalFormatting sqref="A5:I38">
+  <autoFilter ref="A4:I41"/>
+  <conditionalFormatting sqref="A5:I41">
     <cfRule type="expression" priority="1" dxfId="4">
       <formula>$H5="Feito"</formula>
     </cfRule>
@@ -3227,7 +3373,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H5:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Registra o fechamento das inscricoes de 12/10 e o roteiro de 14/10 (AI-002)
DEC-018: prazo de inscricao prorrogado para 12/10 (17 inscritos as 20h),
Jonatas substitui o VIRUS, Junim Reis registra o dia, Agda prepara o
almoco, banner e canecas com valores reais. DEC-019: dinamicas do
amassador de batatas e do sushi no roteiro, despedida depois das 17h
com os QR codes do feedback e do Pix aberto.

Planilha, plano mestre e documentos alinhados; fotos tratadas do Coatio
versionadas apos a aprovacao dele. Dados do Jonatas ainda pendentes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardápio" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$41</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sábado, 17/10/2026 · chegada 10h30, início 11h, fim 17h · Gama/DF · 11 a 20 pessoas no total · inscrições até 10/10 · previsão R$ 500</t>
+          <t>Sábado, 17/10/2026 · chegada 10h30, início 11h, fim 17h · Gama/DF · 11 a 20 pessoas no total · inscrições até 12/10 · previsão R$ 500</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5">
       <c r="A5" s="4" t="n">
         <v>6</v>
       </c>
@@ -676,7 +676,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6">
       <c r="A6" s="4" t="n">
         <v>33</v>
       </c>
@@ -709,7 +709,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7">
       <c r="A7" s="4" t="n">
         <v>34</v>
       </c>
@@ -742,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="90" customHeight="1">
+    <row r="8">
       <c r="A8" s="4" t="n">
         <v>35</v>
       </c>
@@ -775,7 +775,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9">
       <c r="A9" s="4" t="n">
         <v>36</v>
       </c>
@@ -808,7 +808,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1">
+    <row r="10">
       <c r="A10" s="4" t="n">
         <v>40</v>
       </c>
@@ -819,12 +819,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Arthur, Henrique, VIRUS e Coatio se inscreverem no formulário</t>
+          <t>Arthur, Henrique, Coatio e Jonatas se inscreverem no formulário</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Arthur, Henrique, VIRUS e Coatio</t>
+          <t>Arthur, Henrique, Coatio e Jonatas</t>
         </is>
       </c>
       <c r="E10" s="20" t="n">
@@ -832,16 +832,16 @@
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Todos contam nas 20 vagas (DEC-013). Palestrantes até 19/09, confirmado em 15/09 (DEC-016).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t>Todos contam nas 20 vagas (DEC-013). Inscritos em 12/10; Jonatas ocupa o lugar do VIRUS (DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="4" t="n">
         <v>41</v>
       </c>
@@ -874,7 +874,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1">
+    <row r="12">
       <c r="A12" s="4" t="n">
         <v>1</v>
       </c>
@@ -898,16 +898,16 @@
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Telas → sofá → 2 mesas com cadeiras → 2 mesas de plástico extras; quadro de vidro móvel; lanche e café embaixo da escada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+          <t>Uma versão da planta serve; as 3 versões foram dispensadas (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
@@ -940,7 +940,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14">
       <c r="A14" s="4" t="n">
         <v>7</v>
       </c>
@@ -964,51 +964,51 @@
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Coatio entregou em 23/09, dois dias depois do prazo; VIRUS atrasado desde 21/09 (DEC-017). Respostas em docs/evento/RESPOSTAS_PALESTRANTES.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+          <t>Coatio entregou em 23/09; Jonatas tem título, sinopse, minibio e foto com Arthur (12/10). Dados ainda a registrar em docs/evento/RESPOSTAS_PALESTRANTES.md (DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Palestras</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Definir a tela principal: projetor e telão, ou TV</t>
+          <t>Receber o rascunho inicial do material de apoio e uma pergunta para o quiz de cada palestrante</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>TV é o plano B. Sem projetor garantido até esta data, a TV vira a principal. O Coatio pediu projetor + HDMI e tem demonstração do piloto: avisar ele da decisão.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+          <t>Os dois palestrantes entregaram o rascunho e a versão final (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="4" t="n">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Receber o rascunho inicial do material de apoio e uma pergunta para o quiz de cada palestrante</t>
+          <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="E16" s="20" t="n">
-        <v>46293</v>
+        <v>46298</v>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Rascunho até 28/09; versão final e gravação do ensaio até 03/10. Prazos confirmados em 15/09 (DEC-016).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>Os dois palestrantes entregaram a gravação do ensaio com o roteiro (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="4" t="n">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
@@ -1050,45 +1050,45 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
+          <t>Ensaio com a tela escolhida</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Arthur + Henrique + palestrantes</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Ensaio no começo de outubro, gravação com roteiro até 03/10. Confirmado em 15/09 (DEC-016).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>Ensaio feito (12/10). A tela definitiva depende da retirada do projetor (nº 44).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="4" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Separar as mesas de plástico extras, se a planta precisar</t>
+          <t>Brinde: comprar as canecas (2 do sorteio e 2 dos organizadores)</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>Henrique</t>
+          <t>A definir</t>
         </is>
       </c>
       <c r="E18" s="20" t="n">
@@ -1096,28 +1096,32 @@
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>4 canecas mágicas foscas de 325 ml, sublimadas, R$ 209,00 (R$ 52,25 cada, 5% de desconto): 2 do sorteio, 1 de Arthur, 1 de Henrique. Retirada em 24/09. Previsão era 2 por R$ 70 (DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="4" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Testar notebook → cabo/adaptador → tela com material real</t>
+          <t>Confirmar quem prepara e serve o almoço no dia</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E19" s="20" t="n">
@@ -1125,28 +1129,32 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Agda prepara o almoço, arranjo de Henrique (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" s="4" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Palestras</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Ensaio com a tela escolhida</t>
+          <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique + palestrantes</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E20" s="20" t="n">
@@ -1154,32 +1162,32 @@
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Começo de outubro, data a combinar com os palestrantes, junto com o teste da tela (nº 4) (DEC-013).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
+          <t>Proporções prontas (12/10). Conferir contra o número final em 13/10. Aba Cardápio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="4" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Banner: arte e encomenda</t>
+          <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Henrique</t>
         </is>
       </c>
       <c r="E21" s="20" t="n">
@@ -1187,420 +1195,428 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Pedido levantado (12/10). A encomenda sai depois do fechamento, nº 26. Pãezinhos, assados e café.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Inscrições</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Avaliar pedidos de convidados de fora do grupo</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>Não se aplica</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum convidado de fora do grupo pediu entrada até 12/10 (DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Inscrições</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Previsão R$ 60.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Prorrogado de 10/10 para 12/10, 23h59 (DEC-018). 17 inscritos às 20h, 3 vagas livres. Número final em 13/10 na aba Cardápio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Inscrições</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>17 inscritos às 20h de 12/10, 3 vagas livres (DEC-018). Base do aviso de encerramento (Comunicação nº 23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Planejar opção sem lactose e sem glúten para quem informar restrição</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Não se aplica</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Restrição alimentar fica para as próximas edições (DEC-014 e DEC-015). Risco aceito: o cardápio tem glúten e lactose em quase tudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Espaço</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Definir a tela principal: projetor e telão, ou TV</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Projetor emprestado ao Henrique, retirada hoje ou amanhã com um amigo dele (12/10, DEC-018). Decidir depois de retirar; a TV é a reserva. O Coatio pediu projetor + HDMI: avisar na Comunicação nº 37.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Só depois do fechamento da lista (12/10, 23h59). Encomendar com o número final de 13/10 (DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Espaço</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Retirar o projetor emprestado com o amigo do Henrique</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Hoje ou amanhã (DEC-018). Libera a decisão da tela (nº 2), o teste (nº 4) e o aviso ao Coatio (Comunicação nº 37).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Espaço</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Testar notebook → cabo/adaptador → tela com material real</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Depende da retirada do projetor (nº 44). O Coatio precisa de HDMI para a demonstração do piloto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum dos dois está montado (12/10). Arthur monta os dois (DEC-018). docs/evento/SORTEIO_E_FEEDBACK.md + itens de relacionamento do backlog em FORMULARIOS.md. Enviar no encerramento por QR code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Compras</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Brinde: comprar 2 canecas</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Banner: arte e encomenda</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Arte pronta. Fechando a impressão por R$ 54,50 mais entrega, ainda a definir (12/10, DEC-018). Previsão R$ 60.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Espaço</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Separar as mesas de plástico extras, se a planta precisar</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Previsão R$ 70.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Confirmar quem prepara e serve o almoço no dia</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E23" s="20" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Na véspera, 16/10 (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Preparar a dinâmica do amassador de batatas (recepção)</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E24" s="20" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Aba Cardápio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E25" s="20" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Pãezinhos, assados e café.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Inscrições</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Avaliar pedidos de convidados de fora do grupo</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Definida em 14/10 (DEC-019): aproximar as pessoas e deixar o ambiente leve e divertido. Entra no roteiro das 11h às 12h30. Falta descrever o material necessário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Preparar a pergunta de abertura da Mesa 360</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>A pessoa vem com alguém do grupo e também se inscreve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Inscrições</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E27" s="20" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>Anotar o número na aba Cardápio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Inscrições</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="E28" s="20" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Contagem à mão, uma vez por semana a partir do lançamento de 14/09 (DEC-016). Base da peça 5 (últimas vagas).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E29" s="20" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Só depois de 10/10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="4" t="n">
-        <v>39</v>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Planejar opção sem lactose e sem glúten para quem informar restrição</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>Não se aplica</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>Restrição alimentar fica para as próximas edições (DEC-014 e DEC-015). Risco aceito: o cardápio tem glúten e lactose em quase tudo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Dinâmicas</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E31" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md + itens de relacionamento do backlog em FORMULARIOS.md. Enviar no encerramento por QR code ou depois por e-mail/WhatsApp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Dinâmicas</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Preparar a dinâmica de integração da recepção</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E32" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F32" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Aproximar quem estiver isolado e formar grupos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Dinâmicas</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Preparar a pergunta de abertura da Mesa 360</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E33" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Espaço</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
         </is>
       </c>
       <c r="E34" s="20" t="n">
@@ -1611,20 +1627,24 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Na véspera, 16/10 (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
       <c r="A35" s="4" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
+          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
         </is>
       </c>
       <c r="D35" s="14" t="inlineStr">
@@ -1642,58 +1662,218 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Só depois de 10/10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
+          <t>Na véspera, 16/10 (12/10, DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
       <c r="A36" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E36" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Só depois do número final de 13/10 (DEC-018).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Backlog: dinâmica do psiquiatra</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Backlog sem data fixa (DEC-018). Detalhar o que significa ("prev ver relatório clinica") antes de usar. O amassador de batatas e o sushi já entraram no roteiro (nº 29 e 46).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Orçamento</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Decidir com o Henrique como será a dinâmica do QR code de Pix aberto (patron)</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Já conversado com o Henrique em 14/10; falta decidir como fica. Entra na despedida, depois das 17h, junto com o QR do feedback (DEC-019). A participação continua gratuita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Definir o que o Henrique apresenta na Mesa 360 e quanto tempo leva</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Henrique apresenta algo próprio na Mesa 360 (14/10, DEC-019). O assunto e a duração ainda não foram informados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Preparar a dinâmica do sushi para a Mesa 360</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>"Parágrafo de todos, parágrafo de IA": reflexão sobre não domínio, a IA como complemento e não para fazer por você (texto de Arthur). Descrever a mecânica e o material (DEC-019).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Pós-evento</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Fechar o balanço com comprovantes e acertar a divisão</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E36" s="20" t="n">
+      <c r="E41" s="20" t="n">
         <v>46319</v>
       </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="F41" s="14" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>Aba Orçamento.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1"/>
-    <row r="38" ht="30" customHeight="1"/>
-    <row r="39" ht="30" customHeight="1"/>
-    <row r="40" ht="30" customHeight="1"/>
-    <row r="41" ht="30" customHeight="1"/>
     <row r="42" ht="30" customHeight="1"/>
     <row r="43" ht="30" customHeight="1"/>
     <row r="44" ht="30" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A4:G36">
+  <autoFilter ref="A4:G41">
     <sortState ref="A5:G36">
       <sortCondition ref="E4:E36"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A5:G36">
+  <conditionalFormatting sqref="A5:G41">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>$F5="Feito"</formula>
     </cfRule>
@@ -1708,7 +1888,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2214,12 +2394,12 @@
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Encerra a fase só de admins, na noite de 16/09 (DEC-016). Texto pronto em DIVULGACAO.md.</t>
+          <t>Grupo reaberto para todos (confirmado em 12/10).</t>
         </is>
       </c>
     </row>
@@ -2257,12 +2437,12 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Eles contam nas 20 vagas. Libera a cobrança do material.</t>
+          <t>Arthur, Henrique, Coatio e Jonatas inscritos em 12/10 (DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2457,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Convidar Guilherme Reis para registrar o dia, com a peça 1</t>
+          <t>Combinar com Junim Reis o registro do dia (fotos e vídeos)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -2300,12 +2480,12 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Fica 'a confirmar' até ele aceitar.</t>
+          <t>Junim Reis confirmado em 12/10 (DEC-018). Substitui Guilherme Reis, que sai do plano.</t>
         </is>
       </c>
     </row>
@@ -2343,12 +2523,12 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Pessoas próximas, de tecnologia ou de interesse genuíno.</t>
+          <t>Convidados adicionados ao grupo (confirmado em 12/10).</t>
         </is>
       </c>
     </row>
@@ -2386,12 +2566,12 @@
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Coatio respondeu em 23/09, dois dias depois do prazo (DEC-017). VIRUS não respondeu; cobrança na peça 36.</t>
+          <t>Coatio respondeu em 23/09. Jonatas, que substitui o VIRUS, tem os dados com Arthur (12/10, DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2429,12 +2609,12 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Texto, foto tratada em p&amp;b e recorte 4:5 prontos em 23/09 (docs/evento/DIVULGACAO.md e outputs/AI-002/).</t>
+          <t>Coatio aprovou o título curto e a foto tratada (DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2472,12 +2652,12 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Texto pronto em docs/evento/DIVULGACAO.md. A peça 4 não sai antes deste aval (DEC-017).</t>
+          <t>Coatio aprovou o título curto e a foto tratada (12/10, DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2515,12 +2695,12 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Sai como convidado confirmado, sem numerar a palestra, porque o VIRUS ainda não respondeu (DEC-017).</t>
+          <t>Publicado: Coatio anunciado como convidado confirmado (DEC-017). Confirmado por Arthur em 12/10.</t>
         </is>
       </c>
     </row>
@@ -2558,18 +2738,18 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Trava a peça 3 e o anúncio da palestra dele.</t>
+          <t>O VIRUS foi substituído pelo Jonatas (DEC-018).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
@@ -2578,16 +2758,16 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Avisar o Coatio da tela escolhida, projetor ou TV</t>
+          <t>Cobrar o rascunho inicial do material de apresentação</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Decisão de 27/09</t>
+          <t>Título recebido</t>
         </is>
       </c>
       <c r="E23" s="20" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
@@ -2601,18 +2781,18 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Ele pediu projetor + HDMI e tem demonstração do piloto (DEC-017).</t>
+          <t>Os dois palestrantes entregaram o rascunho (12/10).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -2621,16 +2801,16 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Cobrar o rascunho inicial do material de apresentação</t>
+          <t>Combinar o ensaio e cobrar a gravação com o roteiro</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Título recebido</t>
+          <t>Material em rascunho</t>
         </is>
       </c>
       <c r="E24" s="20" t="n">
-        <v>46293</v>
+        <v>46298</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
@@ -2644,18 +2824,18 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Rascunho, não versão final.</t>
+          <t>Ensaio feito e gravações entregues (12/10).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
@@ -2664,16 +2844,16 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Produzir a arte da peça 3 (palestra 1)</t>
+          <t>Produzir a arte da peça 5 (últimas vagas)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Título recebido</t>
+          <t>Vagas em queda</t>
         </is>
       </c>
       <c r="E25" s="20" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
@@ -2687,18 +2867,18 @@
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Parada até o VIRUS responder. Trocou de data com a peça 4 (DEC-017).</t>
+          <t>Absorvida pelo aviso de encerramento, nº 23 (DEC-018).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
@@ -2707,7 +2887,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Anúncio da palestra 1, com a peça 3</t>
+          <t>Últimas vagas, com a peça 5</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -2716,7 +2896,7 @@
         </is>
       </c>
       <c r="E26" s="20" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
@@ -2730,40 +2910,40 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Depende das respostas do VIRUS.</t>
+          <t>Absorvida pelo aviso de encerramento, nº 23 (DEC-018).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>2 · Palestrantes</t>
+          <t>0 · Preparação</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Combinar o ensaio e cobrar a gravação com o roteiro</t>
+          <t>Produzir a arte da peça 3 (palestra 1, Jonatas)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Material em rascunho</t>
+          <t>Título recebido</t>
         </is>
       </c>
       <c r="E27" s="20" t="n">
-        <v>46298</v>
+        <v>46307</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -2778,35 +2958,35 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Junto com o teste da tela.</t>
+          <t>Hoje (DEC-018). Texto em docs/evento/DIVULGACAO.md; falta Arthur enviar os dados do Jonatas ao chat. Arte e envio com os organizadores.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>0 · Preparação</t>
+          <t>3 · Sustentação</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Produzir a arte da peça 5 (últimas vagas)</t>
+          <t>Anúncio da palestra 1 (Jonatas), com a peça 3</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Vagas em queda</t>
+          <t>Arte pronta</t>
         </is>
       </c>
       <c r="E28" s="20" t="n">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="G28" s="14" t="inlineStr">
@@ -2819,11 +2999,15 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I28" s="4" t="n"/>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Hoje, em disparo separado do aviso de encerramento (nº 23) (DEC-018).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -2832,16 +3016,16 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Últimas vagas, com a peça 5</t>
+          <t>Aviso de encerramento das inscrições</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Arte pronta</t>
+          <t>Data-limite</t>
         </is>
       </c>
       <c r="E29" s="20" t="n">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
@@ -2850,7 +3034,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Arthur + Henrique</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
@@ -2860,35 +3044,35 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Precisa do número de vagas restantes.</t>
+          <t>Hoje à noite, em disparo separado da peça 3. 3 vagas livres às 20h; a lista fecha às 23h59 (DEC-018).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>3 · Sustentação</t>
+          <t>4 · Semana do evento</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Aviso de encerramento das inscrições</t>
+          <t>Confirmar presença de cada inscrito</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Data-limite</t>
+          <t>Inscrições encerradas</t>
         </is>
       </c>
       <c r="E30" s="20" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr">
@@ -2903,31 +3087,31 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Última chance de liberar vaga de quem desistir.</t>
+          <t>Mensagem privada a cada inscrito, hoje e ao longo da semana, junto com o lembrete (DEC-018). Base do quantitativo, que fecha em 13/10.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>4 · Semana do evento</t>
+          <t>2 · Palestrantes</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Confirmar presença de cada inscrito</t>
+          <t>Avisar o Coatio da tela escolhida, projetor ou TV</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Inscrições encerradas</t>
+          <t>Decisão de 27/09</t>
         </is>
       </c>
       <c r="E31" s="20" t="n">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
@@ -2936,7 +3120,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Arthur + Henrique</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
@@ -2946,7 +3130,7 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Base do quantitativo de comida.</t>
+          <t>Depois de retirar o projetor (Checklist nº 44), hoje ou amanhã. Ele pediu projetor + HDMI e tem demonstração do piloto (DEC-017).</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3214,11 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I33" s="4" t="n"/>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Inclui o Jonatas. Combinar com o Coatio se o exercício de 2 minutos do fim é no papel ou no celular.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3151,7 +3339,11 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I36" s="4" t="n"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Na despedida, depois das 17h, junto com o QR code do Pix aberto, se confirmado (DEC-019).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3387,7 +3579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="2"/>
@@ -3493,7 +3685,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Check-in, apresentação do dia e das dinâmicas; aproximar quem estiver isolado e formar grupos.</t>
+          <t>Check-in, apresentação do dia (cronograma) e dinâmica do amassador de batatas, conduzida por Arthur, para aproximar as pessoas e deixar o ambiente leve e divertido.</t>
         </is>
       </c>
     </row>
@@ -3515,12 +3707,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Henrique + preparo</t>
+          <t>Henrique + Arthur</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Das 13h30 às 13h45 a equipe prepara o equipamento do VIRUS.</t>
+          <t>Agda prepara o almoço. Das 13h30 às 13h45 a equipe prepara o equipamento do Jonatas.</t>
         </is>
       </c>
     </row>
@@ -3537,17 +3729,17 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Palestra 1 — VIRUS</t>
+          <t>Palestra 1 — Jonatas</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>VIRUS</t>
+          <t>Jonatas</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>IA no dia a dia. Proposta: 30 min de conteúdo + 15 de perguntas.</t>
+          <t>Título e tema a registrar (dados do Jonatas). Proposta: 30 min de conteúdo + 15 de perguntas.</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3783,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Palestra 2 — Coatio</t>
+          <t>Palestra 2 — Matheus Coatio</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -3601,7 +3793,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Design thinking, UI/UX e demonstração do CARANGA.</t>
+          <t>Bastidores do Caranga, demonstração do piloto e exercício de 2 minutos no fim. Precisa de projetor + HDMI.</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3837,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Mesa 360, fechamento e sorteio</t>
+          <t>Mesa 360, sorteio e fechamento</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -3655,23 +3847,45 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Sugestão: Mesa 360 até 16h45; quiz, sorteio das 2 canecas e feedback até 17h.</t>
+          <t>Dinâmica do sushi, sorteio das 2 canecas (quiz por QR code), apresentação do Henrique e fechamento. Duração de cada parte a definir (Checklist nº 45).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Despedida</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Depois do fim oficial das 17h, informal, para quem quiser ficar. QR code do Pix aberto (patron; a dinâmica ainda será decidida) e QR code do formulário de feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C13" s="8">
+      <c r="C14" s="8">
         <f>SUM(C5:C12)</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Se atrasar, encurte a Mesa 360; preserve o almoço e as palestras.</t>
         </is>
@@ -3757,29 +3971,39 @@
       <c r="C5" s="10" t="n"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Agora</t>
+          <t>Até 15/10</t>
         </is>
       </c>
       <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="n"/>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Arte pronta. Fechando por R$ 54,50 mais entrega a definir (12/10); ainda não pago.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Brinde (2 canecas)</t>
+          <t>Brinde (4 canecas)</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="C6" s="10" t="n"/>
+      <c r="C6" s="10" t="n">
+        <v>209</v>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Agora</t>
+          <t>Feito (retirada 24/09)</t>
         </is>
       </c>
       <c r="E6" s="11" t="n"/>
-      <c r="F6" s="11" t="n"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>4 canecas mágicas foscas 325 ml: 2 do sorteio, 1 de Arthur, 1 de Henrique. R$ 52,25 cada. Decidir se as 2 pessoais (R$ 104,50) entram no balanço. Preencher 'Pago por'.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3793,7 +4017,7 @@
       <c r="C7" s="10" t="n"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Depois de 10/10</t>
+          <t>Depois de 12/10</t>
         </is>
       </c>
       <c r="E7" s="11" t="n"/>
@@ -3811,7 +4035,7 @@
       <c r="C8" s="10" t="n"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Depois de 10/10</t>
+          <t>Depois de 12/10</t>
         </is>
       </c>
       <c r="E8" s="11" t="n"/>
@@ -3829,7 +4053,7 @@
       <c r="C9" s="10" t="n"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Depois de 10/10</t>
+          <t>Depois de 12/10</t>
         </is>
       </c>
       <c r="E9" s="11" t="n"/>
@@ -3847,7 +4071,7 @@
       <c r="C10" s="10" t="n"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Depois de 10/10</t>
+          <t>Depois de 12/10</t>
         </is>
       </c>
       <c r="E10" s="11" t="n"/>
@@ -3997,17 +4221,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Henrique preenche as quantidades. Compra só depois de 10/10, com o quantitativo confirmado.</t>
+          <t>Henrique preenche as quantidades. Compra só depois de 12/10, com o quantitativo confirmado.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quantitativo confirmado em 10/10</t>
+          <t>Quantitativo confirmado em 13/10</t>
         </is>
       </c>
       <c r="B4" s="11" t="n"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>17 inscritos às 20h de 12/10; a lista fecha às 23h59. Preencher com o número final.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Registra a vespera e o dia do evento: 20 inscritos, TV e gravacao (AI-002)
DEC-020: inscricoes fechadas em 20, balanco 50/50 com as 4 canecas.
DEC-021: TV como tela principal, banner entregue por R$ 69,90, Pix so
dentro do formulario de feedback, check-in digital pelo QR do banner.

Registra os dados do Jonathan Moura, que nao autorizou gravacao da
palestra, e a orientacao ao fotografo. Novos DIA_DO_EVENTO e DINAMICAS;
quiz e formulario de feedback reescritos; planilha e plano mestre
atualizados. Exportacoes do forms.app ficam fora do commit.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardápio" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$42</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,11 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="&quot;R$&quot; #,##0.00"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -64,16 +61,21 @@
       <sz val="12"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="FF555555"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -95,12 +97,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,9 +126,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -142,19 +141,17 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -164,7 +161,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFDDEBF7"/>
-          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -189,25 +185,25 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00D9EAD3"/>
+          <fgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="00999999"/>
+        <b val="1"/>
+        <color rgb="FFC00000"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <color rgb="00C00000"/>
+        <color rgb="FF999999"/>
       </font>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00DDEBF7"/>
+          <fgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -573,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" customWidth="1" min="1" max="1"/>
@@ -657,15 +653,15 @@
           <t>Enviar o questionário aos dois palestrantes</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="5" t="n">
         <v>46279</v>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -690,15 +686,15 @@
           <t>Criar os formulários online dos palestrantes (VIRUS e Coatio)</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="5" t="n">
         <v>46279</v>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -723,15 +719,15 @@
           <t>Criar o formulário online de inscrição</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="5" t="n">
         <v>46279</v>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -756,15 +752,15 @@
           <t>Revisar e aprovar os 3 formulários antes de enviar ou divulgar</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="5" t="n">
         <v>46281</v>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -789,15 +785,15 @@
           <t>Configurar no formulário o encerramento em 10/10 e o limite de vagas</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="5" t="n">
         <v>46284</v>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
@@ -819,25 +815,25 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Arthur, Henrique, Coatio e Jonatas se inscreverem no formulário</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Arthur, Henrique, Coatio e Jonatas</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="n">
+          <t>Arthur, Henrique, Coatio e Jonathan se inscreverem no formulário</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Arthur, Henrique, Coatio e Jonathan</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
         <v>46284</v>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Todos contam nas 20 vagas (DEC-013). Inscritos em 12/10; Jonatas ocupa o lugar do VIRUS (DEC-018).</t>
+          <t>Todos contam nas 20 vagas (DEC-013). Inscritos em 12/10; Jonathan ocupa o lugar do VIRUS (DEC-018).</t>
         </is>
       </c>
     </row>
@@ -855,15 +851,15 @@
           <t>Aplicar os ajustes pendentes do formulário de inscrição, já em uso</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="5" t="n">
         <v>46284</v>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
@@ -888,15 +884,15 @@
           <t>Desenhar a planta em 3 versões (seca, com móveis, com móveis e pessoas) com os 20 lugares e disponibilizar</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="5" t="n">
         <v>46285</v>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -921,15 +917,15 @@
           <t>Definir como será a inscrição (link ou lista)</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="5" t="n">
         <v>46285</v>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -954,22 +950,22 @@
           <t>Receber títulos e resumos das duas palestras</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="5" t="n">
         <v>46286</v>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Coatio entregou em 23/09; Jonatas tem título, sinopse, minibio e foto com Arthur (12/10). Dados ainda a registrar em docs/evento/RESPOSTAS_PALESTRANTES.md (DEC-018).</t>
+          <t>Coatio entregou em 23/09; Jonathan tem título, sinopse, minibio e foto com Arthur (12/10). Dados ainda a registrar em docs/evento/RESPOSTAS_PALESTRANTES.md (DEC-018).</t>
         </is>
       </c>
     </row>
@@ -987,15 +983,15 @@
           <t>Receber o rascunho inicial do material de apoio e uma pergunta para o quiz de cada palestrante</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="5" t="n">
         <v>46293</v>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1020,15 +1016,15 @@
           <t>Receber a gravação do ensaio com o roteiro de cada palestrante</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="5" t="n">
         <v>46298</v>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1053,15 +1049,15 @@
           <t>Ensaio com a tela escolhida</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique + palestrantes</t>
         </is>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1086,15 +1082,15 @@
           <t>Brinde: comprar as canecas (2 do sorteio e 2 dos organizadores)</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="E18" s="20" t="n">
+      <c r="E18" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1119,15 +1115,15 @@
           <t>Confirmar quem prepara e serve o almoço no dia</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1152,15 +1148,15 @@
           <t>Definir as proporções do almoço para 11, 16 e 20 pessoas</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E20" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1185,15 +1181,15 @@
           <t>Levantar o pedido da padaria para 11, 16 e 20 pessoas</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E21" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -1218,15 +1214,15 @@
           <t>Avaliar pedidos de convidados de fora do grupo</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E22" s="20" t="n">
+      <c r="E22" s="5" t="n">
         <v>46305</v>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
@@ -1251,22 +1247,22 @@
           <t>Encerrar as inscrições e fechar o quantitativo confirmado</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E23" s="20" t="n">
+      <c r="E23" s="5" t="n">
         <v>46307</v>
       </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Prorrogado de 10/10 para 12/10, 23h59 (DEC-018). 17 inscritos às 20h, 3 vagas livres. Número final em 13/10 na aba Cardápio.</t>
+          <t>Fechou com 20 inscritos, lotado (DEC-020). Número anotado na aba Cardápio.</t>
         </is>
       </c>
     </row>
@@ -1284,22 +1280,22 @@
           <t>Acompanhar as inscrições e atualizar a contagem de vagas</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="5" t="n">
         <v>46307</v>
       </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>Em andamento</t>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>17 inscritos às 20h de 12/10, 3 vagas livres (DEC-018). Base do aviso de encerramento (Comunicação nº 23).</t>
+          <t>20 inscritos no fechamento (DEC-020).</t>
         </is>
       </c>
     </row>
@@ -1317,15 +1313,15 @@
           <t>Planejar opção sem lactose e sem glúten para quem informar restrição</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E25" s="20" t="n">
+      <c r="E25" s="5" t="n">
         <v>46307</v>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
@@ -1350,22 +1346,22 @@
           <t>Definir a tela principal: projetor e telão, ou TV</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E26" s="20" t="n">
+      <c r="E26" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>Em andamento</t>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Projetor emprestado ao Henrique, retirada hoje ou amanhã com um amigo dele (12/10, DEC-018). Decidir depois de retirar; a TV é a reserva. O Coatio pediu projetor + HDMI: avisar na Comunicação nº 37.</t>
+          <t>Projetor não retirado; a TV é a tela principal (16/10, DEC-021). Avisar o Coatio: Comunicação nº 37.</t>
         </is>
       </c>
     </row>
@@ -1383,22 +1379,22 @@
           <t>Encomendar o lanche na padaria com o quantitativo confirmado</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E27" s="20" t="n">
+      <c r="E27" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Só depois do fechamento da lista (12/10, 23h59). Encomendar com o número final de 13/10 (DEC-018).</t>
+          <t>Lanche encomendado para 20 pessoas (14/10, DEC-020). Retirada perto das 15h: nº 47.</t>
         </is>
       </c>
     </row>
@@ -1416,160 +1412,160 @@
           <t>Retirar o projetor emprestado com o amigo do Henrique</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E28" s="20" t="n">
+      <c r="E28" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Hoje ou amanhã (DEC-018). Libera a decisão da tela (nº 2), o teste (nº 4) e o aviso ao Coatio (Comunicação nº 37).</t>
+          <t>Projetor não foi retirado; vai a TV (DEC-021).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Testar notebook → cabo/adaptador → tela com material real</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="E29" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+          <t>Banner: arte e encomenda</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Depende da retirada do projetor (nº 44). O Coatio precisa de HDMI para a demonstração do piloto.</t>
+          <t>Banner chegou: R$ 54,90 + R$ 15,00 de entrega = R$ 69,90. Previsão R$ 60 (DEC-021). Tem o QR code do check-in.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Dinâmicas</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+          <t>Separar as mesas de plástico extras, se a planta precisar</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Nenhum dos dois está montado (12/10). Arthur monta os dois (DEC-018). docs/evento/SORTEIO_E_FEEDBACK.md + itens de relacionamento do backlog em FORMULARIOS.md. Enviar no encerramento por QR code.</t>
+          <t>Pronto em 16/10 (DEC-021).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Espaço</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Banner: arte e encomenda</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="E31" s="20" t="n">
-        <v>46310</v>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>Em andamento</t>
+          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Henrique</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Arte pronta. Fechando a impressão por R$ 54,50 mais entrega, ainda a definir (12/10, DEC-018). Previsão R$ 60.</t>
+          <t>Pronto em 16/10 (DEC-021).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Espaço</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Separar as mesas de plástico extras, se a planta precisar</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
+          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E32" s="20" t="n">
+      <c r="E32" s="5" t="n">
         <v>46311</v>
       </c>
-      <c r="F32" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Na véspera, 16/10 (12/10, DEC-018).</t>
+          <t>Compras do almoço prontas em 16/10 (DEC-021). Agda ajudou no preparo e não estará presente.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
@@ -1578,64 +1574,64 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Preparar a dinâmica do amassador de batatas (recepção)</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
+          <t>Backlog: dinâmica do psiquiatra</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E33" s="20" t="n">
+      <c r="E33" s="5" t="n">
         <v>46311</v>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Definida em 14/10 (DEC-019): aproximar as pessoas e deixar o ambiente leve e divertido. Entra no roteiro das 11h às 12h30. Falta descrever o material necessário.</t>
+          <t>Backlog sem data fixa (DEC-018). Detalhar o que significa ("prev ver relatório clinica") antes de usar. O amassador de batatas e o sushi já entraram no roteiro (nº 29 e 46).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Dinâmicas</t>
+          <t>Orçamento</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Preparar a pergunta de abertura da Mesa 360</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="inlineStr">
+          <t>Decidir com o Henrique como será a dinâmica do QR code de Pix aberto (patron)</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E34" s="20" t="n">
+      <c r="E34" s="5" t="n">
         <v>46311</v>
       </c>
-      <c r="F34" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Na véspera, 16/10 (12/10, DEC-018).</t>
+          <t>Arte criada por Arthur; vai só dentro do formulário de feedback, e o valor abate o custo desta edição. Recebedor não informado (DEC-021).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
@@ -1644,64 +1640,64 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Posicionar 2 ou 3 ventiladores cruzados na sala e testar</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E35" s="20" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F35" s="14" t="inlineStr">
+          <t>Testar notebook → cabo/adaptador → tela com material real</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Na véspera, 16/10 (12/10, DEC-018).</t>
+          <t>Na TV, na manhã de 17/10 ou às 13h30 (Jonathan) e 13h45 (Coatio). O Coatio precisa de HDMI para a demonstração do piloto.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Comprar ingredientes do almoço, refrigerantes, sucos e café</t>
-        </is>
-      </c>
-      <c r="D36" s="14" t="inlineStr">
-        <is>
-          <t>Henrique</t>
-        </is>
-      </c>
-      <c r="E36" s="20" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F36" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+          <t>Montar o quiz do QR code e o formulário de feedback e relacionamento</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Só depois do número final de 13/10 (DEC-018).</t>
+          <t>Em 16/10 nenhum estava pronto; Arthur monta com o conteúdo de docs/evento/SORTEIO_E_FEEDBACK.md. Gerar os QR codes e testar pelo celular (DEC-021).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
@@ -1710,58 +1706,58 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Backlog: dinâmica do psiquiatra</t>
-        </is>
-      </c>
-      <c r="D37" s="14" t="inlineStr">
+          <t>Preparar a dinâmica do amassador de batatas (recepção)</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E37" s="20" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F37" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="E37" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Backlog sem data fixa (DEC-018). Detalhar o que significa ("prev ver relatório clinica") antes de usar. O amassador de batatas e o sushi já entraram no roteiro (nº 29 e 46).</t>
+          <t>Amassador de batatas quase pronto em 16/10; Arthur está finalizando (DEC-021). Descrição em docs/evento/DINAMICAS.md quando fechar.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Orçamento</t>
+          <t>Dinâmicas</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Decidir com o Henrique como será a dinâmica do QR code de Pix aberto (patron)</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
+          <t>Preparar a pergunta de abertura da Mesa 360</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E38" s="20" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F38" s="14" t="inlineStr">
-        <is>
-          <t>Em andamento</t>
+      <c r="E38" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Já conversado com o Henrique em 14/10; falta decidir como fica. Entra na despedida, depois das 17h, junto com o QR do feedback (DEC-019). A participação continua gratuita.</t>
+          <t>Adiada da véspera. Mesa 360: 15 min sushi, 10 apresentação do Henrique, 5 quiz, 5 sorteio, 10 fechamento (DEC-021).</t>
         </is>
       </c>
     </row>
@@ -1779,26 +1775,26 @@
           <t>Definir o que o Henrique apresenta na Mesa 360 e quanto tempo leva</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="E39" s="20" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F39" s="14" t="inlineStr">
+      <c r="E39" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Henrique apresenta algo próprio na Mesa 360 (14/10, DEC-019). O assunto e a duração ainda não foram informados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
+          <t>Tempo aceito em 16/10: 10 min na Mesa 360. O assunto segue a anunciar (DEC-021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40" s="4" t="n">
         <v>46</v>
       </c>
@@ -1812,83 +1808,179 @@
           <t>Preparar a dinâmica do sushi para a Mesa 360</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="E40" s="20" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F40" s="14" t="inlineStr">
+      <c r="E40" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>"Parágrafo de todos, parágrafo de IA": reflexão sobre não domínio, a IA como complemento e não para fazer por você (texto de Arthur). Descrever a mecânica e o material (DEC-019).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
+          <t>Backlog por último (16/10). A IA vem depois das pessoas. Decidir o tema antes das 16h15 e guardar a resposta da IA. Roteiro em docs/evento/DINAMICAS.md (DEC-021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Retirar o lanche encomendado na padaria, perto das 15h</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>O responsável não foi informado (16/10). O lanche é servido às 15h45 (DEC-021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Inscrições</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Testar o QR code do check-in no banner com o celular, com a lista do painel do forms.app como reserva</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Fazer antes das 10h30. Se a rede cair, usar a lista do painel (DEC-021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Divulgação</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Orientar o Junim Reis: fotos podem, mas NÃO gravar áudio nem vídeo da palestra do Jonathan</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Jonathan não autorizou gravação (formulário dele). O Coatio autorizou fotos e gravação, com divulgação pública mediante aprovação dele (DEC-021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Pós-evento</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Fechar o balanço com comprovantes e acertar a divisão</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
+      <c r="D44" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E41" s="20" t="n">
+      <c r="E44" s="5" t="n">
         <v>46319</v>
       </c>
-      <c r="F41" s="14" t="inlineStr">
+      <c r="F44" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>Aba Orçamento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1"/>
-    <row r="43" ht="30" customHeight="1"/>
-    <row r="44" ht="30" customHeight="1"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Tudo dividido 50/50 depois do evento (DEC-020). Entram as 4 canecas (R$ 209,00), o banner (R$ 69,90) e o Pix recebido, que abate o custo. Aba Orçamento.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G41">
+  <autoFilter ref="A4:G44">
     <sortState ref="A5:G36">
       <sortCondition ref="E4:E36"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A5:G41">
-    <cfRule type="expression" priority="5" dxfId="4">
+  <conditionalFormatting sqref="A5:G44">
+    <cfRule type="expression" priority="5" dxfId="3">
       <formula>$F5="Feito"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="5">
+    <cfRule type="expression" priority="6" dxfId="2">
       <formula>$F5="Não se aplica"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="6">
+    <cfRule type="expression" priority="7" dxfId="1">
       <formula>AND($E5&lt;TODAY(),$F5&lt;&gt;"Feito",$F5&lt;&gt;"Não se aplica")</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="7">
+    <cfRule type="expression" priority="8" dxfId="0">
       <formula>$F5="Aguardando aprovação"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1903,7 +1995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1917,15 +2009,15 @@
     <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>TECHNE Talks · Encontro nº 02 — comunicação</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Ordem padrão das mensagens, reutilizável nas próximas edições. Passo a passo e radar do que ainda falta comunicar: docs/evento/COMUNICACAO.md. Textos prontos: docs/evento/DIVULGACAO.md.</t>
         </is>
@@ -1939,47 +2031,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Nº</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Peça / mensagem</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Gatilho</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Canal</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>Responsável</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
@@ -2004,7 +2096,7 @@
           <t>Data e local fechados</t>
         </is>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="5" t="n">
         <v>46277</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -2012,12 +2104,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2043,7 +2135,7 @@
           <t>Identidade fechada</t>
         </is>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -2051,12 +2143,12 @@
           <t>Repositório</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2086,7 +2178,7 @@
           <t>Textos prontos</t>
         </is>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -2094,12 +2186,12 @@
           <t>forms.app</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2129,7 +2221,7 @@
           <t>Textos aprovados</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2137,12 +2229,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2168,7 +2260,7 @@
           <t>Artes prontas</t>
         </is>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -2176,12 +2268,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2211,7 +2303,7 @@
           <t>Aprovação</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -2219,12 +2311,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H10" s="14" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2254,7 +2346,7 @@
           <t>Antes do disparo</t>
         </is>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -2262,12 +2354,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2297,7 +2389,7 @@
           <t>Grupo preparado</t>
         </is>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -2305,12 +2397,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2340,7 +2432,7 @@
           <t>Formulário aprovado</t>
         </is>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="5" t="n">
         <v>46279</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2348,12 +2440,12 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G13" s="14" t="inlineStr">
+      <c r="G13" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2379,7 +2471,7 @@
           <t>Primeira rodada absorvida</t>
         </is>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="5" t="n">
         <v>46281</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -2387,12 +2479,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2422,7 +2514,7 @@
           <t>Questionário enviado</t>
         </is>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="5" t="n">
         <v>46284</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -2430,19 +2522,19 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Arthur, Henrique, Coatio e Jonatas inscritos em 12/10 (DEC-018).</t>
+          <t>Arthur, Henrique, Coatio e Jonathan inscritos em 12/10 (DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2557,7 @@
           <t>Peça 1 publicada</t>
         </is>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="5" t="n">
         <v>46286</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -2473,12 +2565,12 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>Henrique</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2508,7 +2600,7 @@
           <t>Lançamento feito</t>
         </is>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="5" t="n">
         <v>46286</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2516,12 +2608,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2551,7 +2643,7 @@
           <t>Inscrição confirmada</t>
         </is>
       </c>
-      <c r="E18" s="20" t="n">
+      <c r="E18" s="5" t="n">
         <v>46286</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -2559,19 +2651,19 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="G18" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="H18" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Coatio respondeu em 23/09. Jonatas, que substitui o VIRUS, tem os dados com Arthur (12/10, DEC-018).</t>
+          <t>Coatio respondeu em 23/09. Jonathan, que substitui o VIRUS, tem os dados com Arthur (12/10, DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2686,7 @@
           <t>Título recebido</t>
         </is>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="5" t="n">
         <v>46289</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2602,12 +2694,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G19" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2637,7 +2729,7 @@
           <t>Respostas recebidas</t>
         </is>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E20" s="5" t="n">
         <v>46289</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2645,12 +2737,12 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr">
+      <c r="G20" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H20" s="14" t="inlineStr">
+      <c r="H20" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2680,7 +2772,7 @@
           <t>Arte pronta</t>
         </is>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E21" s="5" t="n">
         <v>46290</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2688,12 +2780,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
+      <c r="G21" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="H21" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2723,7 +2815,7 @@
           <t>Prazo vencido em 21/09</t>
         </is>
       </c>
-      <c r="E22" s="20" t="n">
+      <c r="E22" s="5" t="n">
         <v>46291</v>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2731,19 +2823,19 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="G22" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="H22" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>O VIRUS foi substituído pelo Jonatas (DEC-018).</t>
+          <t>O VIRUS foi substituído pelo Jonathan (DEC-018).</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2858,7 @@
           <t>Título recebido</t>
         </is>
       </c>
-      <c r="E23" s="20" t="n">
+      <c r="E23" s="5" t="n">
         <v>46293</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2774,12 +2866,12 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="G23" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H23" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2809,7 +2901,7 @@
           <t>Material em rascunho</t>
         </is>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="5" t="n">
         <v>46298</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2817,12 +2909,12 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="G24" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H24" s="14" t="inlineStr">
+      <c r="H24" s="13" t="inlineStr">
         <is>
           <t>Feito</t>
         </is>
@@ -2852,7 +2944,7 @@
           <t>Vagas em queda</t>
         </is>
       </c>
-      <c r="E25" s="20" t="n">
+      <c r="E25" s="5" t="n">
         <v>46300</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -2860,12 +2952,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G25" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H25" s="14" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
@@ -2895,7 +2987,7 @@
           <t>Arte pronta</t>
         </is>
       </c>
-      <c r="E26" s="20" t="n">
+      <c r="E26" s="5" t="n">
         <v>46301</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -2903,12 +2995,12 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="G26" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H26" s="13" t="inlineStr">
         <is>
           <t>Não se aplica</t>
         </is>
@@ -2930,7 +3022,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Produzir a arte da peça 3 (palestra 1, Jonatas)</t>
+          <t>Produzir a arte da peça 3 (palestra 1, Jonathan)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -2938,7 +3030,7 @@
           <t>Título recebido</t>
         </is>
       </c>
-      <c r="E27" s="20" t="n">
+      <c r="E27" s="5" t="n">
         <v>46307</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2946,19 +3038,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="14" t="inlineStr">
+      <c r="G27" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H27" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Hoje (DEC-018). Texto em docs/evento/DIVULGACAO.md; falta Arthur enviar os dados do Jonatas ao chat. Arte e envio com os organizadores.</t>
+          <t>Arte e texto criados por Arthur; peça 3 publicada (confirmado em 14/10, DEC-020).</t>
         </is>
       </c>
     </row>
@@ -2973,7 +3065,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Anúncio da palestra 1 (Jonatas), com a peça 3</t>
+          <t>Anúncio da palestra 1 (Jonathan), com a peça 3</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -2981,7 +3073,7 @@
           <t>Arte pronta</t>
         </is>
       </c>
-      <c r="E28" s="20" t="n">
+      <c r="E28" s="5" t="n">
         <v>46307</v>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -2989,19 +3081,19 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="G28" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H28" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Hoje, em disparo separado do aviso de encerramento (nº 23) (DEC-018).</t>
+          <t>Anúncio da palestra 1 enviado, em disparo separado do aviso de encerramento (14/10, DEC-020).</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3116,7 @@
           <t>Data-limite</t>
         </is>
       </c>
-      <c r="E29" s="20" t="n">
+      <c r="E29" s="5" t="n">
         <v>46307</v>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3032,19 +3124,19 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G29" s="14" t="inlineStr">
+      <c r="G29" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H29" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Hoje à noite, em disparo separado da peça 3. 3 vagas livres às 20h; a lista fecha às 23h59 (DEC-018).</t>
+          <t>Aviso de encerramento enviado (14/10, DEC-020).</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3159,7 @@
           <t>Inscrições encerradas</t>
         </is>
       </c>
-      <c r="E30" s="20" t="n">
+      <c r="E30" s="5" t="n">
         <v>46307</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3075,19 +3167,19 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
+      <c r="G30" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H30" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Mensagem privada a cada inscrito, hoje e ao longo da semana, junto com o lembrete (DEC-018). Base do quantitativo, que fecha em 13/10.</t>
+          <t>Mensagem privada a cada inscrito (DEC-018). Usar o check-in digital para ver quem não respondeu.</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3202,7 @@
           <t>Decisão de 27/09</t>
         </is>
       </c>
-      <c r="E31" s="20" t="n">
+      <c r="E31" s="5" t="n">
         <v>46309</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -3118,19 +3210,19 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G31" s="14" t="inlineStr">
+      <c r="G31" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H31" s="14" t="inlineStr">
+      <c r="H31" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Depois de retirar o projetor (Checklist nº 44), hoje ou amanhã. Ele pediu projetor + HDMI e tem demonstração do piloto (DEC-017).</t>
+          <t>A TV é a tela (DEC-021). Texto pronto em DIVULGACAO.md ('Aviso da tela ao Coatio'). Enviar se ainda não saiu.</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3245,7 @@
           <t>Presença confirmada</t>
         </is>
       </c>
-      <c r="E32" s="20" t="n">
+      <c r="E32" s="5" t="n">
         <v>46310</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -3161,19 +3253,19 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G32" s="14" t="inlineStr">
+      <c r="G32" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="H32" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>O endereço já está na peça 1; o lembrete reforça e confirma.</t>
+          <t>Arte com cronograma no grupo e texto em docs/evento/DIVULGACAO.md ('Lembrete final no grupo'). Enviar se ainda não saiu.</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3288,7 @@
           <t>Ensaio feito</t>
         </is>
       </c>
-      <c r="E33" s="20" t="n">
+      <c r="E33" s="5" t="n">
         <v>46310</v>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -3204,64 +3296,68 @@
           <t>Privado</t>
         </is>
       </c>
-      <c r="G33" s="14" t="inlineStr">
+      <c r="G33" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H33" s="14" t="inlineStr">
-        <is>
-          <t>A fazer</t>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Inclui o Jonatas. Combinar com o Coatio se o exercício de 2 minutos do fim é no papel ou no celular.</t>
+          <t>Roteiro e horários confirmados com os palestrantes (14/10, DEC-020).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>5 · Dia</t>
+          <t>4 · Semana do evento</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Bom dia com endereço e horário de chegada</t>
+          <t>Lembrete aos palestrantes: chegar até 12h45 e testar o equipamento</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Manhã do evento</t>
-        </is>
-      </c>
-      <c r="E34" s="20" t="n">
-        <v>46312</v>
+          <t>Roteiro confirmado</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>46311</v>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="inlineStr">
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
         <is>
           <t>Arthur</t>
         </is>
       </c>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="H34" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I34" s="4" t="n"/>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Testes às 13h30 (Jonathan) e 13h45 (Coatio). Texto em docs/evento/DIVULGACAO.md (DEC-021).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
@@ -3270,41 +3366,37 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Divulgar o QR code do quiz e conduzir o sorteio</t>
+          <t>Bom dia com endereço e horário de chegada</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Mesa 360</t>
-        </is>
-      </c>
-      <c r="E35" s="20" t="n">
+          <t>Manhã do evento</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
         <v>46312</v>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>No local</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="H35" s="14" t="inlineStr">
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
-        </is>
-      </c>
+      <c r="I35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
@@ -3313,15 +3405,15 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Divulgar o QR code do feedback no encerramento</t>
+          <t>Divulgar o QR code do quiz e conduzir o sorteio</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Encerramento</t>
-        </is>
-      </c>
-      <c r="E36" s="20" t="n">
+          <t>Mesa 360</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
         <v>46312</v>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -3329,64 +3421,68 @@
           <t>No local</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G36" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H36" s="14" t="inlineStr">
+      <c r="H36" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Na despedida, depois das 17h, junto com o QR code do Pix aberto, se confirmado (DEC-019).</t>
+          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>6 · Pós-evento</t>
+          <t>5 · Dia</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Agradecimento no grupo, no mesmo dia</t>
+          <t>Divulgar o QR code do feedback no encerramento</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Fim do evento</t>
-        </is>
-      </c>
-      <c r="E37" s="20" t="n">
+          <t>Encerramento</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
         <v>46312</v>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="H37" s="14" t="inlineStr">
+          <t>No local</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I37" s="4" t="n"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Na despedida, depois das 17h, o QR code do feedback. O Pix fica dentro do formulário, sem QR na tela (DEC-021).</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
@@ -3395,41 +3491,37 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Publicar fotos e materiais autorizados</t>
+          <t>Agradecimento no grupo, no mesmo dia</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Autorizações conferidas</t>
-        </is>
-      </c>
-      <c r="E38" s="20" t="n">
-        <v>46315</v>
+          <t>Fim do evento</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>46312</v>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="G38" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="H38" s="14" t="inlineStr">
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>Só o que palestrantes e participantes autorizaram.</t>
-        </is>
-      </c>
+      <c r="I38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
@@ -3438,37 +3530,41 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Reenviar o feedback a quem não respondeu</t>
+          <t>Publicar fotos e materiais autorizados</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Respostas paradas</t>
-        </is>
-      </c>
-      <c r="E39" s="20" t="n">
+          <t>Autorizações conferidas</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
         <v>46315</v>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Privado</t>
-        </is>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="H39" s="14" t="inlineStr">
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I39" s="4" t="n"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Só o que palestrantes e participantes autorizaram.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
@@ -3477,28 +3573,28 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Resultado do feedback e convite para a próxima edição</t>
+          <t>Reenviar o feedback a quem não respondeu</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Feedback consolidado</t>
-        </is>
-      </c>
-      <c r="E40" s="20" t="n">
-        <v>46319</v>
+          <t>Respostas paradas</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>46315</v>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>Arthur + Henrique</t>
-        </is>
-      </c>
-      <c r="H40" s="14" t="inlineStr">
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
@@ -3507,65 +3603,104 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>6 · Pós-evento</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Resultado do feedback e convite para a próxima edição</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Feedback consolidado</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>Arthur + Henrique</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>6 · Pós-evento</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Registrar os aprendizados de comunicação da edição</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Contas fechadas</t>
         </is>
       </c>
-      <c r="E41" s="20" t="n">
+      <c r="E42" s="5" t="n">
         <v>46319</v>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>Repositório</t>
         </is>
       </c>
-      <c r="G41" s="14" t="inlineStr">
+      <c r="G42" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="H41" s="14" t="inlineStr">
+      <c r="H42" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>O que mudar no passo a passo da próxima edição.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I41"/>
-  <conditionalFormatting sqref="A5:I41">
-    <cfRule type="expression" priority="1" dxfId="4">
+  <autoFilter ref="A4:I42"/>
+  <conditionalFormatting sqref="A5:I42">
+    <cfRule type="expression" priority="1" dxfId="3">
       <formula>$H5="Feito"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="5">
+    <cfRule type="expression" priority="2" dxfId="2">
       <formula>$H5="Não se aplica"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="6">
+    <cfRule type="expression" priority="3" dxfId="1">
       <formula>AND($E5&lt;TODAY(),$H5&lt;&gt;"Feito",$H5&lt;&gt;"Não se aplica")</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="7">
+    <cfRule type="expression" priority="4" dxfId="0">
       <formula>$H5="Aguardando aprovação"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3582,27 +3717,29 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="34.42578125" customWidth="1" min="1" max="1"/>
+    <col width="6" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="29.85546875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="17" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="79" bestFit="1" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Roteiro do dia — 17/10</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Equipe arruma o espaço antes das 10h30 e desmonta depois das 17h.</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3636,10 +3773,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>0.4375</v>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="6" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="C5">
@@ -3658,15 +3795,15 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Horário divulgado. Equipe já arrumou o espaço; água disponível.</t>
+          <t>Horário divulgado. Equipe já arrumou o espaço; água disponível. Check-in digital pelo QR code do banner.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="6" t="n">
         <v>0.5208333333333334</v>
       </c>
       <c r="C6">
@@ -3689,11 +3826,11 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="6" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="C7">
@@ -3712,15 +3849,15 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Agda prepara o almoço. Das 13h30 às 13h45 a equipe prepara o equipamento do Jonatas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n">
+          <t>Agda ajudou no preparo e não estará presente. Testes de equipamento na TV: 13h30 com o Jonathan e 13h45 com o Coatio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="6" t="n">
         <v>0.6145833333333334</v>
       </c>
       <c r="C8">
@@ -3729,25 +3866,25 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Palestra 1 — Jonatas</t>
+          <t>Palestra 1 — Jonathan Moura</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Jonatas</t>
+          <t>Jonathan Moura</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Título e tema a registrar (dados do Jonatas). Proposta: 30 min de conteúdo + 15 de perguntas.</t>
+          <t>O Estado da IA em 2026 (State of AI Report 2026). Só slides, sem demonstração; perguntas só ao final. Fotos sim; gravação NÃO autorizada. 30 min de conteúdo + 15 de perguntas.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>0.6145833333333334</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="6" t="n">
         <v>0.625</v>
       </c>
       <c r="C9">
@@ -3770,11 +3907,11 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="6" t="n">
         <v>0.65625</v>
       </c>
       <c r="C10">
@@ -3793,15 +3930,15 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Bastidores do Caranga, demonstração do piloto e exercício de 2 minutos no fim. Precisa de projetor + HDMI.</t>
+          <t>Bastidores do Caranga, demonstração do piloto na TV (HDMI) e exercício de 2 minutos no fim. Fotos e gravação autorizadas; divulgação pública só com aprovação dele.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>0.65625</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="6" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="C11">
@@ -3825,10 +3962,10 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
       <c r="C12">
@@ -3847,15 +3984,15 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Dinâmica do sushi, sorteio das 2 canecas (quiz por QR code), apresentação do Henrique e fechamento. Duração de cada parte a definir (Checklist nº 45).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+          <t>Sushi 15 min (a IA depois das pessoas), apresentação do Henrique 10, quiz 5, sorteio e resultado 5, fechamento 10 (DEC-021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="6" t="n"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Despedida</t>
@@ -3868,17 +4005,17 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Depois do fim oficial das 17h, informal, para quem quiser ficar. QR code do Pix aberto (patron; a dinâmica ainda será decidida) e QR code do formulário de feedback.</t>
+          <t>Depois do fim oficial das 17h, informal, para quem quiser ficar. QR code do formulário de feedback; o Pix aparece só dentro do formulário (DEC-021).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="7">
         <f>SUM(C5:C12)</f>
         <v/>
       </c>
@@ -3927,6 +4064,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3965,19 +4103,21 @@
           <t>Banner</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="C5" s="10" t="n"/>
+      <c r="C5" s="9" t="n">
+        <v>69.90000000000001</v>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Até 15/10</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Arte pronta. Fechando por R$ 54,50 mais entrega a definir (12/10); ainda não pago.</t>
+          <t>Feito (chegou)</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>R$ 54,90 + R$ 15,00 de entrega = R$ 69,90. Previsão R$ 60 (DEC-021). Preencher 'Pago por'.</t>
         </is>
       </c>
     </row>
@@ -3987,10 +4127,10 @@
           <t>Brinde (4 canecas)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="9" t="n">
         <v>209</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -3998,10 +4138,10 @@
           <t>Feito (retirada 24/09)</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>4 canecas mágicas foscas 325 ml: 2 do sorteio, 1 de Arthur, 1 de Henrique. R$ 52,25 cada. Decidir se as 2 pessoais (R$ 104,50) entram no balanço. Preencher 'Pago por'.</t>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>4 canecas mágicas foscas 325 ml: 2 do sorteio, 1 de Arthur, 1 de Henrique. R$ 52,25 cada. As 4 entram no balanço 50/50 (DEC-020). Preencher 'Pago por'.</t>
         </is>
       </c>
     </row>
@@ -4011,17 +4151,17 @@
           <t>Almoço</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>250</v>
       </c>
-      <c r="C7" s="10" t="n"/>
+      <c r="C7" s="9" t="n"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Depois de 12/10</t>
         </is>
       </c>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4029,17 +4169,21 @@
           <t>Lanche</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="C8" s="10" t="n"/>
+      <c r="C8" s="9" t="n"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Depois de 12/10</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
+          <t>Encomendado (valor a lançar)</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Encomendado para 20 pessoas (14/10). Retirada perto das 15h. Lançar o valor real e quem pagou.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4047,17 +4191,17 @@
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="C9" s="10" t="n"/>
+      <c r="C9" s="9" t="n"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Depois de 12/10</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4065,36 +4209,36 @@
           <t>Café</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="C10" s="10" t="n"/>
+      <c r="C10" s="9" t="n"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Depois de 12/10</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Soma</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="11">
         <f>SUM(B5:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="11">
         <f>SUM(C5:C10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
     </row>
     <row r="13" ht="18.75" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
@@ -4102,8 +4246,8 @@
           <t>Balanço</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4111,10 +4255,10 @@
           <t>Previsão da edição</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="C14" s="9" t="n"/>
+      <c r="C14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4122,11 +4266,11 @@
           <t>Soma das categorias − previsão</t>
         </is>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="8">
         <f>B11-B14</f>
         <v/>
       </c>
-      <c r="C15" s="9" t="n"/>
+      <c r="C15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4134,11 +4278,11 @@
           <t>Gasto real total</t>
         </is>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <f>C11</f>
         <v/>
       </c>
-      <c r="C16" s="9" t="n"/>
+      <c r="C16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4146,11 +4290,11 @@
           <t>Pago por Arthur</t>
         </is>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <f>SUMIF(E5:E10,"Arthur",C5:C10)</f>
         <v/>
       </c>
-      <c r="C17" s="9" t="n"/>
+      <c r="C17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4158,11 +4302,11 @@
           <t>Pago por Henrique</t>
         </is>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <f>SUMIF(E5:E10,"Henrique",C5:C10)</f>
         <v/>
       </c>
-      <c r="C18" s="9" t="n"/>
+      <c r="C18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4170,11 +4314,11 @@
           <t>Parte de cada um (metade)</t>
         </is>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <f>C11/2</f>
         <v/>
       </c>
-      <c r="C19" s="9" t="n"/>
+      <c r="C19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4182,7 +4326,7 @@
           <t>Acerto: positivo = Henrique repassa a Arthur</t>
         </is>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="8">
         <f>B17-B19</f>
         <v/>
       </c>
@@ -4225,16 +4369,19 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Quantitativo confirmado em 13/10</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n"/>
+      <c r="B4" s="10" t="n">
+        <v>20</v>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>17 inscritos às 20h de 12/10; a lista fecha às 23h59. Preencher com o número final.</t>
+          <t>20 inscritos, lotado (DEC-020). Agda não estará presente; o Junim está entre os 20.</t>
         </is>
       </c>
     </row>
@@ -4249,8 +4396,9 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Almoço</t>
         </is>
@@ -4294,17 +4442,17 @@
           <t>Lasanha</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>travessa</t>
         </is>
       </c>
-      <c r="F9" s="11" t="n"/>
+      <c r="F9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4312,11 +4460,11 @@
           <t>Estrogonofe</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4324,11 +4472,11 @@
           <t>Arroz</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4336,11 +4484,11 @@
           <t>Batata palha</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4348,11 +4496,11 @@
           <t>Salada</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4360,11 +4508,11 @@
           <t>Refrigerante</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4372,14 +4520,16 @@
           <t>Suco</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-    </row>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Lanche (padaria)</t>
         </is>
@@ -4423,11 +4573,11 @@
           <t>Pãezinhos</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4435,11 +4585,11 @@
           <t>Assados</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4447,11 +4597,11 @@
           <t>Café</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Registra a roleta do sorteio e os lembretes enviados (AI-002)
DEC-022: o quiz do forms.app saiu da edicao; as 2 canecas sao sorteadas
por uma roleta em HTML com quiz (10 min na Mesa 360). Formulario de
feedback e QR codes criados, QR do check-in testado, avisos enviados.

Documenta o uso da roleta e um defeito conhecido do botao de adicionar
pessoa (sem id); o arquivo nao foi alterado. Planilha com nome dos
participantes fica fora do commit.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI-002/planejamento-evento.xlsx
+++ b/outputs/AI-002/planejamento-evento.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardápio" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$4:$G$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comunicação'!$A$4:$I$42</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" customWidth="1" min="1" max="1"/>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Em 16/10 nenhum estava pronto; Arthur monta com o conteúdo de docs/evento/SORTEIO_E_FEEDBACK.md. Gerar os QR codes e testar pelo celular (DEC-021).</t>
+          <t>Formulário de feedback criado e QR codes criados (17/10). O quiz do forms.app foi removido da edição; o sorteio usa a roleta (DEC-022).</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Adiada da véspera. Mesa 360: 15 min sushi, 10 apresentação do Henrique, 5 quiz, 5 sorteio, 10 fechamento (DEC-021).</t>
+          <t>Adiada da véspera. Mesa 360: sushi 15 min, apresentação do Henrique 10, roleta com quiz 10, fechamento 10 (DEC-022).</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
       </c>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Fazer antes das 10h30. Se a rede cair, usar a lista do painel (DEC-021).</t>
+          <t>QR code do check-in testado (17/10, DEC-022). Lista do painel do forms.app como reserva.</t>
         </is>
       </c>
     </row>
@@ -1928,44 +1928,77 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Dinâmicas</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Preparar a roleta do sorteio no telão: importar o check-in, desmarcar organizadores e palestrantes e testar o giro</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F44" s="13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Arquivo roleta/TECHNE_Talks_Roleta_Sorteio.html, offline. Não usar '+ Adicionar pessoa' com 2 ou mais nomes (defeito de identificação, ver DEC-022). Abrir já com a lista importada (DEC-022).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>Pós-evento</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Fechar o balanço com comprovantes e acertar a divisão</t>
         </is>
       </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="D45" s="13" t="inlineStr">
         <is>
           <t>Arthur + Henrique</t>
         </is>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E45" s="5" t="n">
         <v>46319</v>
       </c>
-      <c r="F44" s="13" t="inlineStr">
+      <c r="F45" s="13" t="inlineStr">
         <is>
           <t>A fazer</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>Tudo dividido 50/50 depois do evento (DEC-020). Entram as 4 canecas (R$ 209,00), o banner (R$ 69,90) e o Pix recebido, que abate o custo. Aba Orçamento.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G44">
+  <autoFilter ref="A4:G45">
     <sortState ref="A5:G36">
       <sortCondition ref="E4:E36"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A5:G44">
+  <conditionalFormatting sqref="A5:G45">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>$F5="Feito"</formula>
     </cfRule>
@@ -1980,7 +2013,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A fazer,Em andamento,Feito,Aguardando aprovação,Não se aplica"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3217,12 +3250,12 @@
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>A TV é a tela (DEC-021). Texto pronto em DIVULGACAO.md ('Aviso da tela ao Coatio'). Enviar se ainda não saiu.</t>
+          <t>Aviso da TV ao Coatio enviado (confirmado em 17/10, DEC-022).</t>
         </is>
       </c>
     </row>
@@ -3260,12 +3293,12 @@
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Arte com cronograma no grupo e texto em docs/evento/DIVULGACAO.md ('Lembrete final no grupo'). Enviar se ainda não saiu.</t>
+          <t>Lembrete final no grupo, com a arte, enviado em 16/10 ou 17/10 (confirmado por Arthur em 17/10, DEC-022).</t>
         </is>
       </c>
     </row>
@@ -3346,12 +3379,12 @@
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Testes às 13h30 (Jonathan) e 13h45 (Coatio). Texto em docs/evento/DIVULGACAO.md (DEC-021).</t>
+          <t>Lembrete aos palestrantes enviado (confirmado em 17/10, DEC-022).</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3425,11 @@
           <t>A fazer</t>
         </is>
       </c>
-      <c r="I35" s="4" t="n"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Sai hoje cedo (17/10, DEC-022).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3405,7 +3442,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Divulgar o QR code do quiz e conduzir o sorteio</t>
+          <t>Conduzir o sorteio das 2 canecas pela roleta com quiz, no telão</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -3433,7 +3470,7 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>docs/evento/SORTEIO_E_FEEDBACK.md</t>
+          <t>Sem QR code de quiz: a roleta roda na TV (DEC-022). 10 min na Mesa 360.</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3776,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3984,7 +4020,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Sushi 15 min (a IA depois das pessoas), apresentação do Henrique 10, quiz 5, sorteio e resultado 5, fechamento 10 (DEC-021).</t>
+          <t>Sushi 15 min (a IA depois das pessoas), apresentação do Henrique 10, roleta com quiz 10 (sorteio das 2 canecas), fechamento 10 (DEC-022).</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4056,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -4064,7 +4099,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4369,7 +4403,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -4396,7 +4429,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
@@ -4526,8 +4558,6 @@
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="10" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>

</xml_diff>